<commit_message>
Session 2026-08-29: WO-P000-E2.001/E3.001/E12.001 closed, E2.003/E4.002/E19.001 built, WO_COMPLETION_GATE.md Ack Scope rule added, peh-handoff v1.9, P_005 nested-repo fix
</commit_message>
<xml_diff>
--- a/projects/P_010_Current_Market_Posture/data/excel_exports/History Grid (VXX)_v3.xlsx
+++ b/projects/P_010_Current_Market_Posture/data/excel_exports/History Grid (VXX)_v3.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="27">
   <si>
     <t>High
 Price</t>
@@ -67,11 +67,11 @@
 Price</t>
   </si>
   <si>
-    <t>Medium</t>
+    <t>Low
+Price</t>
   </si>
   <si>
-    <t>Low
-Price</t>
+    <t>Triple Cross Medium</t>
   </si>
   <si>
     <t>Long
@@ -81,9 +81,6 @@
   <si>
     <t>Close
 Price</t>
-  </si>
-  <si>
-    <t>Long</t>
   </si>
   <si>
     <t>Predicted
@@ -96,9 +93,6 @@
 Difference</t>
   </si>
   <si>
-    <t>Short</t>
-  </si>
-  <si>
     <t>Volume</t>
   </si>
   <si>
@@ -108,11 +102,17 @@
     <t>ROC%</t>
   </si>
   <si>
+    <t>Triple Cross Short</t>
+  </si>
+  <si>
     <t>Williams
 EMAI</t>
   </si>
   <si>
     <t>Neural Index</t>
+  </si>
+  <si>
+    <t>Triple Cross Long</t>
   </si>
 </sst>
 </file>
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V44"/>
+  <dimension ref="A1:V45"/>
   <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="13.85546875" customWidth="1"/>
@@ -466,9 +466,9 @@
     <col min="14" max="14" width="17.28515625" customWidth="1"/>
     <col min="15" max="15" width="12.85546875" customWidth="1"/>
     <col min="16" max="16" width="17.7109375" customWidth="1"/>
-    <col min="17" max="17" width="10" customWidth="1"/>
-    <col min="18" max="18" width="13.28515625" customWidth="1"/>
-    <col min="19" max="19" width="9.5703125" customWidth="1"/>
+    <col min="17" max="17" width="23.7109375" customWidth="1"/>
+    <col min="18" max="18" width="27" customWidth="1"/>
+    <col min="19" max="19" width="23.28515625" customWidth="1"/>
     <col min="20" max="22" width="14.5703125" customWidth="1"/>
     <col min="23" max="16384" width="8.7265625"/>
   </cols>
@@ -481,7 +481,7 @@
         <v>12</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>16</v>
@@ -493,28 +493,28 @@
         <v>0</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>17</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="K1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M1" t="s">
         <v>9</v>
       </c>
       <c r="O1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="Q1" t="s">
         <v>3</v>
@@ -544,7 +544,7 @@
         <v>4</v>
       </c>
       <c r="N2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="O2" t="s">
         <v>10</v>
@@ -553,13 +553,13 @@
         <v>8</v>
       </c>
       <c r="Q2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="R2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="S2" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="T2" s="1"/>
       <c r="U2" s="1"/>
@@ -567,1631 +567,1631 @@
     </row>
     <row r="3" ht="19.5" customHeight="1">
       <c r="A3" s="2">
-        <v>46247</v>
+        <v>46261</v>
       </c>
       <c r="B3">
-        <v>-0.113121032714844</v>
+        <v>-0.276155471801758</v>
       </c>
       <c r="C3">
-        <v>-0.529033660888672</v>
+        <v>-0.314380645751953</v>
       </c>
       <c r="D3">
-        <v>-1.04665374755859</v>
+        <v>-0.566484451293945</v>
       </c>
       <c r="E3">
-        <v>19.3999996185303</v>
+        <v>18.5100002288818</v>
       </c>
       <c r="F3">
-        <v>19.7099990844727</v>
+        <v>18.5799999237061</v>
       </c>
       <c r="G3">
-        <v>19.3600006103516</v>
+        <v>18.0650005340576</v>
       </c>
       <c r="H3">
-        <v>19.6200008392334</v>
+        <v>18.1000003814697</v>
       </c>
       <c r="I3">
-        <v>19.9825096130371</v>
+        <v>18.8255252838135</v>
       </c>
       <c r="J3">
-        <v>19.7475090026855</v>
+        <v>17.7851409912109</v>
       </c>
       <c r="K3">
-        <v>6271200</v>
+        <v>7733800</v>
       </c>
       <c r="L3">
-        <v>-0.054047629237175</v>
+        <v>-0.147857114672661</v>
       </c>
       <c r="M3">
-        <v>49.7687377929688</v>
+        <v>74.4601974487305</v>
       </c>
       <c r="N3">
-        <v>11.6717119216919</v>
+        <v>21.4995422363281</v>
       </c>
       <c r="O3" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="P3">
-        <v>36.0380020141602</v>
+        <v>-21.5595436096191</v>
       </c>
       <c r="Q3">
-        <v>19.9000854492188</v>
+        <v>18.4563503265381</v>
       </c>
       <c r="R3">
-        <v>20.354133605957</v>
+        <v>18.9632472991943</v>
       </c>
       <c r="S3">
-        <v>20.9163265228271</v>
+        <v>19.5502548217773</v>
       </c>
       <c r="T3">
-        <v>0.272510528564453</v>
+        <v>0.245525360107422</v>
       </c>
       <c r="U3">
-        <v>0.387508392333984</v>
+        <v>-0.27985954284668</v>
       </c>
       <c r="V3">
-        <v>0.235000610351563</v>
+        <v>1.04038429260254</v>
       </c>
     </row>
     <row r="4" ht="19.5" customHeight="1">
       <c r="A4" s="2">
-        <v>46246</v>
+        <v>46260</v>
       </c>
       <c r="B4">
-        <v>-0.167993545532227</v>
+        <v>-0.232177734375</v>
       </c>
       <c r="C4">
-        <v>-0.525745391845703</v>
+        <v>-0.297714233398438</v>
       </c>
       <c r="D4">
-        <v>-1.00045394897461</v>
+        <v>-0.549018859863281</v>
       </c>
       <c r="E4">
-        <v>19.8700008392334</v>
+        <v>18.6900005340576</v>
       </c>
       <c r="F4">
-        <v>19.9200000762939</v>
+        <v>18.7649993896484</v>
       </c>
       <c r="G4">
-        <v>19.4200000762939</v>
+        <v>18.5200004577637</v>
       </c>
       <c r="H4">
-        <v>19.4500007629395</v>
+        <v>18.5400009155273</v>
       </c>
       <c r="I4">
-        <v>19.9356956481934</v>
+        <v>19.1796894073486</v>
       </c>
       <c r="J4">
-        <v>19.7006950378418</v>
+        <v>18.1763000488281</v>
       </c>
       <c r="K4">
-        <v>7554400</v>
+        <v>4331500</v>
       </c>
       <c r="L4">
-        <v>-0.0816666707396507</v>
+        <v>-0.0773809552192688</v>
       </c>
       <c r="M4">
-        <v>44.5670051574707</v>
+        <v>61.2843437194824</v>
       </c>
       <c r="N4">
-        <v>13.1198835372925</v>
+        <v>16.0765419006348</v>
       </c>
       <c r="O4" t="s">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="P4">
-        <v>-6.83822298049927</v>
+        <v>18.9501953125</v>
       </c>
       <c r="Q4">
-        <v>20.0184288024902</v>
+        <v>18.6757259368896</v>
       </c>
       <c r="R4">
-        <v>20.5874538421631</v>
+        <v>19.1171398162842</v>
       </c>
       <c r="S4">
-        <v>21.0807361602783</v>
+        <v>19.6962242126465</v>
       </c>
       <c r="T4">
-        <v>0.0156955718994141</v>
+        <v>0.414690017700195</v>
       </c>
       <c r="U4">
-        <v>0.280694961547852</v>
+        <v>-0.343700408935547</v>
       </c>
       <c r="V4">
-        <v>0.235000610351563</v>
+        <v>1.00338935852051</v>
       </c>
     </row>
     <row r="5" ht="19.5" customHeight="1">
       <c r="A5" s="2">
-        <v>46245</v>
+        <v>46259</v>
       </c>
       <c r="B5">
-        <v>-0.00268936157226563</v>
+        <v>-0.338632583618164</v>
       </c>
       <c r="C5">
-        <v>-0.60869026184082</v>
+        <v>-0.178274154663086</v>
       </c>
       <c r="D5">
-        <v>-0.90032958984375</v>
+        <v>-0.528701782226563</v>
       </c>
       <c r="E5">
-        <v>20.2299995422363</v>
+        <v>18.7999992370605</v>
       </c>
       <c r="F5">
-        <v>20.3150005340576</v>
+        <v>19.0324993133545</v>
       </c>
       <c r="G5">
-        <v>20.0499992370605</v>
+        <v>18.6200008392334</v>
       </c>
       <c r="H5">
-        <v>20.0499992370605</v>
+        <v>18.6700000762939</v>
       </c>
       <c r="I5">
-        <v>20.3811225891113</v>
+        <v>19.1117668151855</v>
       </c>
       <c r="J5">
-        <v>20.1461219787598</v>
+        <v>17.7509269714355</v>
       </c>
       <c r="K5">
-        <v>5997000</v>
+        <v>5731700</v>
       </c>
       <c r="L5">
-        <v>-0.0583333522081375</v>
+        <v>-0.0780952125787735</v>
       </c>
       <c r="M5">
-        <v>39.3980293273926</v>
+        <v>52.7964935302734</v>
       </c>
       <c r="N5">
-        <v>2.98054528236389</v>
+        <v>-19.5024471282959</v>
       </c>
       <c r="O5" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="P5">
-        <v>10.9317674636841</v>
+        <v>-14.6816358566284</v>
       </c>
       <c r="Q5">
-        <v>20.3394374847412</v>
+        <v>18.7199401855469</v>
       </c>
       <c r="R5">
-        <v>20.862621307373</v>
+        <v>19.2823104858398</v>
       </c>
       <c r="S5">
-        <v>21.2543029785156</v>
+        <v>19.8400802612305</v>
       </c>
       <c r="T5">
-        <v>0.0661220550537109</v>
+        <v>0.0792675018310547</v>
       </c>
       <c r="U5">
-        <v>0.0961227416992188</v>
+        <v>-0.869073867797852</v>
       </c>
       <c r="V5">
-        <v>0.235000610351563</v>
+        <v>1.36083984375</v>
       </c>
     </row>
     <row r="6" ht="19.5" customHeight="1">
       <c r="A6" s="2">
-        <v>46244</v>
+        <v>46258</v>
       </c>
       <c r="B6">
-        <v>-0.10870361328125</v>
+        <v>-0.305706024169922</v>
       </c>
       <c r="C6">
-        <v>-0.670436859130859</v>
+        <v>-0.312480926513672</v>
       </c>
       <c r="D6">
-        <v>-0.835453033447266</v>
+        <v>-0.63226318359375</v>
       </c>
       <c r="E6">
-        <v>20.2399997711182</v>
+        <v>18.8199996948242</v>
       </c>
       <c r="F6">
-        <v>20.2999992370605</v>
+        <v>19.0100002288818</v>
       </c>
       <c r="G6">
-        <v>20.0200004577637</v>
+        <v>18.7849998474121</v>
       </c>
       <c r="H6">
-        <v>20.2099990844727</v>
+        <v>18.9599990844727</v>
       </c>
       <c r="I6">
-        <v>20.5593681335449</v>
+        <v>19.1353855133057</v>
       </c>
       <c r="J6">
-        <v>20.2264862060547</v>
+        <v>18.4291210174561</v>
       </c>
       <c r="K6">
-        <v>6569000</v>
+        <v>6196100</v>
       </c>
       <c r="L6">
-        <v>-0.0297619048506021</v>
+        <v>-0.0519048608839512</v>
       </c>
       <c r="M6">
-        <v>38.257740020752</v>
+        <v>65.5876998901367</v>
       </c>
       <c r="N6">
-        <v>-0.424057513475418</v>
+        <v>-28.9931240081787</v>
       </c>
       <c r="O6" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="P6">
-        <v>95.0116653442383</v>
+        <v>-12.4073457717896</v>
       </c>
       <c r="Q6">
-        <v>20.4868125915527</v>
+        <v>18.9291191101074</v>
       </c>
       <c r="R6">
-        <v>21.0531120300293</v>
+        <v>19.3523998260498</v>
       </c>
       <c r="S6">
-        <v>21.3902626037598</v>
+        <v>19.941349029541</v>
       </c>
       <c r="T6">
-        <v>0.259368896484375</v>
+        <v>0.125385284423828</v>
       </c>
       <c r="U6">
-        <v>0.206485748291016</v>
+        <v>-0.355878829956055</v>
       </c>
       <c r="V6">
-        <v>0.332881927490234</v>
+        <v>0.706264495849609</v>
       </c>
     </row>
     <row r="7" ht="19.5" customHeight="1">
       <c r="A7" s="2">
-        <v>46241</v>
+        <v>46255</v>
       </c>
       <c r="B7">
-        <v>-0.14726448059082</v>
+        <v>-0.388160705566406</v>
       </c>
       <c r="C7">
-        <v>-0.642946243286133</v>
+        <v>-0.277084350585938</v>
       </c>
       <c r="D7">
-        <v>-0.803007125854492</v>
+        <v>-0.630989074707031</v>
       </c>
       <c r="E7">
-        <v>20.2600002288818</v>
+        <v>18.9500007629395</v>
       </c>
       <c r="F7">
-        <v>20.4150009155273</v>
+        <v>19.0499992370605</v>
       </c>
       <c r="G7">
-        <v>20.1800003051758</v>
+        <v>18.8700008392334</v>
       </c>
       <c r="H7">
-        <v>20.3199996948242</v>
+        <v>18.9500007629395</v>
       </c>
       <c r="I7">
-        <v>20.7853908538818</v>
+        <v>18.9418525695801</v>
       </c>
       <c r="J7">
-        <v>20.0895118713379</v>
+        <v>18.1200313568115</v>
       </c>
       <c r="K7">
-        <v>6660500</v>
+        <v>6056600</v>
       </c>
       <c r="L7">
-        <v>-0.0459523871541023</v>
+        <v>-0.0661905407905579</v>
       </c>
       <c r="M7">
-        <v>38.4206657409668</v>
+        <v>92.3680953979492</v>
       </c>
       <c r="N7">
-        <v>-10.2513265609741</v>
+        <v>25.1085910797119</v>
       </c>
       <c r="O7" t="s">
         <v>1</v>
       </c>
       <c r="P7">
-        <v>15.8023986816406</v>
+        <v>2.40918016433716</v>
       </c>
       <c r="Q7">
-        <v>20.6419906616211</v>
+        <v>19.0168037414551</v>
       </c>
       <c r="R7">
-        <v>21.3021640777588</v>
+        <v>19.4948863983154</v>
       </c>
       <c r="S7">
-        <v>21.527416229248</v>
+        <v>20.0736389160156</v>
       </c>
       <c r="T7">
-        <v>0.370389938354492</v>
+        <v>-0.108146667480469</v>
       </c>
       <c r="U7">
-        <v>-0.0904884338378906</v>
+        <v>-0.749969482421875</v>
       </c>
       <c r="V7">
-        <v>0.695878982543945</v>
+        <v>0.821821212768555</v>
       </c>
     </row>
     <row r="8" ht="19.5" customHeight="1">
       <c r="A8" s="2">
-        <v>46240</v>
+        <v>46254</v>
       </c>
       <c r="B8">
-        <v>-0.0613174438476563</v>
+        <v>-0.0505161285400391</v>
       </c>
       <c r="C8">
-        <v>-0.548988342285156</v>
+        <v>-0.243555068969727</v>
       </c>
       <c r="D8">
-        <v>-0.691572189331055</v>
+        <v>-0.579545974731445</v>
       </c>
       <c r="E8">
-        <v>20.7000007629395</v>
+        <v>19.2299995422363</v>
       </c>
       <c r="F8">
-        <v>20.7399997711182</v>
+        <v>19.3899993896484</v>
       </c>
       <c r="G8">
-        <v>20.2049999237061</v>
+        <v>19.0904998779297</v>
       </c>
       <c r="H8">
-        <v>20.2299995422363</v>
+        <v>19.1900005340576</v>
       </c>
       <c r="I8">
-        <v>21.2324962615967</v>
+        <v>20.5423545837402</v>
       </c>
       <c r="J8">
-        <v>20.8165054321289</v>
+        <v>18.3230438232422</v>
       </c>
       <c r="K8">
-        <v>5901700</v>
+        <v>9287900</v>
       </c>
       <c r="L8">
-        <v>-0.0621428713202477</v>
+        <v>-0.0766666978597641</v>
       </c>
       <c r="M8">
-        <v>42.8091735839844</v>
+        <v>73.8303375244141</v>
       </c>
       <c r="N8">
-        <v>48.3031349182129</v>
+        <v>2.45110702514648</v>
       </c>
       <c r="O8" t="s">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="P8">
-        <v>-4.02017259597778</v>
+        <v>30.8698177337646</v>
       </c>
       <c r="Q8">
-        <v>20.8864498138428</v>
+        <v>19.3633308410645</v>
       </c>
       <c r="R8">
-        <v>21.5750007629395</v>
+        <v>19.6456489562988</v>
       </c>
       <c r="S8">
-        <v>21.6811447143555</v>
+        <v>20.244140625</v>
       </c>
       <c r="T8">
-        <v>0.492496490478516</v>
+        <v>1.1523551940918</v>
       </c>
       <c r="U8">
-        <v>0.611505508422852</v>
+        <v>-0.7674560546875</v>
       </c>
       <c r="V8">
-        <v>0.415990829467773</v>
+        <v>2.21931076049805</v>
       </c>
     </row>
     <row r="9" ht="19.5" customHeight="1">
       <c r="A9" s="2">
-        <v>46239</v>
+        <v>46253</v>
       </c>
       <c r="B9">
-        <v>-0.285120010375977</v>
+        <v>-0.243087768554688</v>
       </c>
       <c r="C9">
-        <v>-0.137289047241211</v>
+        <v>-0.387598037719727</v>
       </c>
       <c r="D9">
-        <v>-0.377473831176758</v>
+        <v>-0.755746841430664</v>
       </c>
       <c r="E9">
-        <v>21.3400001525879</v>
+        <v>19.3799991607666</v>
       </c>
       <c r="F9">
-        <v>21.4400005340576</v>
+        <v>19.4300003051758</v>
       </c>
       <c r="G9">
-        <v>20.3799991607666</v>
+        <v>18.9799995422363</v>
       </c>
       <c r="H9">
-        <v>20.5100002288818</v>
+        <v>19.0499992370605</v>
       </c>
       <c r="I9">
-        <v>21.4269924163818</v>
+        <v>19.1709480285645</v>
       </c>
       <c r="J9">
-        <v>20.5687198638916</v>
+        <v>18.2612934112549</v>
       </c>
       <c r="K9">
-        <v>11253400</v>
+        <v>7460400</v>
       </c>
       <c r="L9">
-        <v>-0.0469047017395496</v>
+        <v>-0.0771429911255836</v>
       </c>
       <c r="M9">
-        <v>28.8659934997559</v>
+        <v>72.0639724731445</v>
       </c>
       <c r="N9">
-        <v>38.9394416809082</v>
+        <v>4.47362422943115</v>
       </c>
       <c r="O9" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="P9">
-        <v>99.9001083374023</v>
+        <v>-37.1015090942383</v>
       </c>
       <c r="Q9">
-        <v>21.0118141174316</v>
+        <v>19.3749351501465</v>
       </c>
       <c r="R9">
-        <v>21.9915046691895</v>
+        <v>19.7025089263916</v>
       </c>
       <c r="S9">
-        <v>21.8754062652588</v>
+        <v>20.3463687896729</v>
       </c>
       <c r="T9">
-        <v>-0.0130081176757813</v>
+        <v>-0.259052276611328</v>
       </c>
       <c r="U9">
-        <v>0.188720703125</v>
+        <v>-0.718706130981445</v>
       </c>
       <c r="V9">
-        <v>0.858272552490234</v>
+        <v>0.90965461730957</v>
       </c>
     </row>
     <row r="10" ht="19.5" customHeight="1">
       <c r="A10" s="2">
-        <v>46238</v>
+        <v>46252</v>
       </c>
       <c r="B10">
-        <v>-0.735685348510742</v>
+        <v>0.405941009521484</v>
       </c>
       <c r="C10">
-        <v>0.0724983215332031</v>
+        <v>-0.348033905029297</v>
       </c>
       <c r="D10">
-        <v>-0.173707962036133</v>
+        <v>-0.828088760375977</v>
       </c>
       <c r="E10">
-        <v>20.7700004577637</v>
+        <v>19.7099990844727</v>
       </c>
       <c r="F10">
-        <v>21.2700004577637</v>
+        <v>19.75</v>
       </c>
       <c r="G10">
-        <v>20.7696990966797</v>
+        <v>19.5200004577637</v>
       </c>
       <c r="H10">
-        <v>21.2700004577637</v>
+        <v>19.6499996185303</v>
       </c>
       <c r="I10">
-        <v>21.6324405670166</v>
+        <v>20.141429901123</v>
       </c>
       <c r="J10">
-        <v>19.8532638549805</v>
+        <v>19.9114303588867</v>
       </c>
       <c r="K10">
-        <v>7316800</v>
+        <v>8474900</v>
       </c>
       <c r="L10">
-        <v>0.00214295159094036</v>
+        <v>-0.0742857828736305</v>
       </c>
       <c r="M10">
-        <v>20.7759532928467</v>
+        <v>68.9781494140625</v>
       </c>
       <c r="N10">
-        <v>-12.7948808670044</v>
+        <v>-9.15783214569092</v>
       </c>
       <c r="O10" t="s">
         <v>1</v>
       </c>
       <c r="P10">
-        <v>49.2009391784668</v>
+        <v>47.6022415161133</v>
       </c>
       <c r="Q10">
-        <v>21.1883125305176</v>
+        <v>19.9225387573242</v>
       </c>
       <c r="R10">
-        <v>22.2094955444336</v>
+        <v>19.8831005096436</v>
       </c>
       <c r="S10">
-        <v>21.9951305389404</v>
+        <v>20.521411895752</v>
       </c>
       <c r="T10">
-        <v>0.36244010925293</v>
+        <v>0.391429901123047</v>
       </c>
       <c r="U10">
-        <v>-0.916435241699219</v>
+        <v>0.391429901123047</v>
       </c>
       <c r="V10">
-        <v>1.77917671203613</v>
+        <v>0.229999542236328</v>
       </c>
     </row>
     <row r="11" ht="19.5" customHeight="1">
       <c r="A11" s="2">
-        <v>46237</v>
+        <v>46251</v>
       </c>
       <c r="B11">
-        <v>-0.65983772277832</v>
+        <v>0.366083145141602</v>
       </c>
       <c r="C11">
-        <v>0.0400638580322266</v>
+        <v>-0.402734756469727</v>
       </c>
       <c r="D11">
-        <v>-0.0176563262939453</v>
+        <v>-0.883899688720703</v>
       </c>
       <c r="E11">
-        <v>21.0699996948242</v>
+        <v>19.3500003814697</v>
       </c>
       <c r="F11">
-        <v>21.1800003051758</v>
+        <v>19.7000007629395</v>
       </c>
       <c r="G11">
-        <v>20.8950004577637</v>
+        <v>19.2800006866455</v>
       </c>
       <c r="H11">
-        <v>21.0799999237061</v>
+        <v>19.5</v>
       </c>
       <c r="I11">
-        <v>21.4725818634033</v>
+        <v>20.5525894165039</v>
       </c>
       <c r="J11">
-        <v>20.4887065887451</v>
+        <v>20.0624809265137</v>
       </c>
       <c r="K11">
-        <v>6825100</v>
+        <v>8042800</v>
       </c>
       <c r="L11">
-        <v>-0.0326189324259758</v>
+        <v>-0.0514286570250988</v>
       </c>
       <c r="M11">
-        <v>23.8242359161377</v>
+        <v>75.9318618774414</v>
       </c>
       <c r="N11">
-        <v>-17.6793479919434</v>
+        <v>53.9863471984863</v>
       </c>
       <c r="O11" t="s">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="P11">
-        <v>-61.7687721252441</v>
+        <v>36.4534568786621</v>
       </c>
       <c r="Q11">
-        <v>21.4585494995117</v>
+        <v>19.9442195892334</v>
       </c>
       <c r="R11">
-        <v>22.2541065216064</v>
+        <v>20.0184993743896</v>
       </c>
       <c r="S11">
-        <v>22.0823230743408</v>
+        <v>20.6447105407715</v>
       </c>
       <c r="T11">
-        <v>0.292581558227539</v>
+        <v>0.852588653564453</v>
       </c>
       <c r="U11">
-        <v>-0.406293869018555</v>
+        <v>0.782480239868164</v>
       </c>
       <c r="V11">
-        <v>0.983875274658203</v>
+        <v>0.490108489990234</v>
       </c>
     </row>
     <row r="12" ht="19.5" customHeight="1">
       <c r="A12" s="2">
-        <v>46234</v>
+        <v>46248</v>
       </c>
       <c r="B12">
-        <v>-0.393699645996094</v>
+        <v>0.0695743560791016</v>
       </c>
       <c r="C12">
-        <v>0.704631805419922</v>
+        <v>-0.549312591552734</v>
       </c>
       <c r="D12">
-        <v>0.512554168701172</v>
+        <v>-1.01874351501465</v>
       </c>
       <c r="E12">
-        <v>21.6399993896484</v>
+        <v>19.4400005340576</v>
       </c>
       <c r="F12">
-        <v>22.5100002288818</v>
+        <v>19.6200008392334</v>
       </c>
       <c r="G12">
-        <v>21.1800003051758</v>
+        <v>19.3199996948242</v>
       </c>
       <c r="H12">
-        <v>21.25</v>
+        <v>19.3549995422363</v>
       </c>
       <c r="I12">
-        <v>22.9274063110352</v>
+        <v>20.1421585083008</v>
       </c>
       <c r="J12">
-        <v>20.3054065704346</v>
+        <v>19.9071578979492</v>
       </c>
       <c r="K12">
-        <v>8503300</v>
+        <v>5526100</v>
       </c>
       <c r="L12">
-        <v>-0.0340474434196949</v>
+        <v>-0.0719048604369164</v>
       </c>
       <c r="M12">
-        <v>28.9407768249512</v>
+        <v>49.3107757568359</v>
       </c>
       <c r="N12">
-        <v>28.6269283294678</v>
+        <v>-0.920180141925812</v>
       </c>
       <c r="O12" t="s">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="P12">
-        <v>-22.4164390563965</v>
+        <v>12.46812915802</v>
       </c>
       <c r="Q12">
-        <v>21.9039173126221</v>
+        <v>19.8505516052246</v>
       </c>
       <c r="R12">
-        <v>22.6548538208008</v>
+        <v>20.1270999908447</v>
       </c>
       <c r="S12">
-        <v>22.2817363739014</v>
+        <v>20.7514057159424</v>
       </c>
       <c r="T12">
-        <v>0.41740608215332</v>
+        <v>0.522157669067383</v>
       </c>
       <c r="U12">
-        <v>-0.874593734741211</v>
+        <v>0.587158203125</v>
       </c>
       <c r="V12">
-        <v>2.62199974060059</v>
+        <v>0.235000610351563</v>
       </c>
     </row>
     <row r="13" ht="19.5" customHeight="1">
       <c r="A13" s="2">
-        <v>46233</v>
+        <v>46247</v>
       </c>
       <c r="B13">
-        <v>-0.0996761322021484</v>
+        <v>-0.113121032714844</v>
       </c>
       <c r="C13">
-        <v>1.02289772033691</v>
+        <v>-0.529033660888672</v>
       </c>
       <c r="D13">
-        <v>0.774198532104492</v>
+        <v>-1.04665374755859</v>
       </c>
       <c r="E13">
-        <v>22.4799995422363</v>
+        <v>19.3999996185303</v>
       </c>
       <c r="F13">
-        <v>22.7700004577637</v>
+        <v>19.7099990844727</v>
       </c>
       <c r="G13">
-        <v>21.8199996948242</v>
+        <v>19.3600006103516</v>
       </c>
       <c r="H13">
-        <v>21.8199996948242</v>
+        <v>19.6200008392334</v>
       </c>
       <c r="I13">
-        <v>23.2930679321289</v>
+        <v>19.9825096130371</v>
       </c>
       <c r="J13">
-        <v>20.6710681915283</v>
+        <v>19.7475090026855</v>
       </c>
       <c r="K13">
-        <v>9302900</v>
+        <v>6271200</v>
       </c>
       <c r="L13">
-        <v>-0.0169046483933926</v>
+        <v>-0.054047629237175</v>
       </c>
       <c r="M13">
-        <v>22.4997806549072</v>
+        <v>49.7687377929688</v>
       </c>
       <c r="N13">
-        <v>300.6494140625</v>
+        <v>11.6717119216919</v>
       </c>
       <c r="O13" t="s">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="P13">
-        <v>-31.0044631958008</v>
+        <v>36.0380020141602</v>
       </c>
       <c r="Q13">
-        <v>22.3125190734863</v>
+        <v>19.9000854492188</v>
       </c>
       <c r="R13">
-        <v>22.8138961791992</v>
+        <v>20.354133605957</v>
       </c>
       <c r="S13">
-        <v>22.3450241088867</v>
+        <v>20.9163265228271</v>
       </c>
       <c r="T13">
-        <v>0.523067474365234</v>
+        <v>0.272510528564453</v>
       </c>
       <c r="U13">
-        <v>-1.1489315032959</v>
+        <v>0.387508392333984</v>
       </c>
       <c r="V13">
-        <v>2.62199974060059</v>
+        <v>0.235000610351563</v>
       </c>
     </row>
     <row r="14" ht="19.5" customHeight="1">
       <c r="A14" s="2">
-        <v>46232</v>
+        <v>46246</v>
       </c>
       <c r="B14">
-        <v>0.441112518310547</v>
+        <v>-0.167993545532227</v>
       </c>
       <c r="C14">
-        <v>0.785587310791016</v>
+        <v>-0.525745391845703</v>
       </c>
       <c r="D14">
-        <v>0.695182800292969</v>
+        <v>-1.00045394897461</v>
       </c>
       <c r="E14">
-        <v>22.3500003814697</v>
+        <v>19.8700008392334</v>
       </c>
       <c r="F14">
-        <v>23.5100002288818</v>
+        <v>19.9200000762939</v>
       </c>
       <c r="G14">
-        <v>21.7950000762939</v>
+        <v>19.4200000762939</v>
       </c>
       <c r="H14">
-        <v>23.4200000762939</v>
+        <v>19.4500007629395</v>
       </c>
       <c r="I14">
-        <v>24.9417915344238</v>
+        <v>19.9356956481934</v>
       </c>
       <c r="J14">
-        <v>22.3197937011719</v>
+        <v>19.7006950378418</v>
       </c>
       <c r="K14">
-        <v>18832500</v>
+        <v>7554400</v>
       </c>
       <c r="L14">
-        <v>-0.00976181030273438</v>
+        <v>-0.0816666707396507</v>
       </c>
       <c r="M14">
-        <v>5.61582803726196</v>
+        <v>44.5670051574707</v>
       </c>
       <c r="N14">
-        <v>-80.1277160644531</v>
+        <v>13.1198835372925</v>
       </c>
       <c r="O14" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="P14">
-        <v>64.2163772583008</v>
+        <v>-6.83822298049927</v>
       </c>
       <c r="Q14">
-        <v>22.6965599060059</v>
+        <v>20.0184288024902</v>
       </c>
       <c r="R14">
-        <v>22.5893497467041</v>
+        <v>20.5874538421631</v>
       </c>
       <c r="S14">
-        <v>22.2805633544922</v>
+        <v>21.0807361602783</v>
       </c>
       <c r="T14">
-        <v>1.43179130554199</v>
+        <v>0.0156955718994141</v>
       </c>
       <c r="U14">
-        <v>0.52479362487793</v>
+        <v>0.280694961547852</v>
       </c>
       <c r="V14">
-        <v>2.62199783325195</v>
+        <v>0.235000610351563</v>
       </c>
     </row>
     <row r="15" ht="19.5" customHeight="1">
       <c r="A15" s="2">
-        <v>46231</v>
+        <v>46245</v>
       </c>
       <c r="B15">
-        <v>-0.407449722290039</v>
+        <v>-0.00268936157226563</v>
       </c>
       <c r="C15">
-        <v>0.318998336791992</v>
+        <v>-0.60869026184082</v>
       </c>
       <c r="D15">
-        <v>0.211315155029297</v>
+        <v>-0.90032958984375</v>
       </c>
       <c r="E15">
-        <v>22.1949996948242</v>
+        <v>20.2299995422363</v>
       </c>
       <c r="F15">
-        <v>22.5599994659424</v>
+        <v>20.3150005340576</v>
       </c>
       <c r="G15">
-        <v>21.8250007629395</v>
+        <v>20.0499992370605</v>
       </c>
       <c r="H15">
-        <v>22.0300006866455</v>
+        <v>20.0499992370605</v>
       </c>
       <c r="I15">
-        <v>21.4767627716064</v>
+        <v>20.3811225891113</v>
       </c>
       <c r="J15">
-        <v>21.1667633056641</v>
+        <v>20.1461219787598</v>
       </c>
       <c r="K15">
-        <v>6852400</v>
+        <v>5997000</v>
       </c>
       <c r="L15">
-        <v>-0.0754761472344398</v>
+        <v>-0.0583333522081375</v>
       </c>
       <c r="M15">
-        <v>28.2595958709717</v>
+        <v>39.3980293273926</v>
       </c>
       <c r="N15">
-        <v>-6.67150163650513</v>
+        <v>2.98054528236389</v>
       </c>
       <c r="O15" t="s">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="P15">
-        <v>-20.5401268005371</v>
+        <v>10.9317674636841</v>
       </c>
       <c r="Q15">
-        <v>21.8332195281982</v>
+        <v>20.3394374847412</v>
       </c>
       <c r="R15">
-        <v>22.1766109466553</v>
+        <v>20.862621307373</v>
       </c>
       <c r="S15">
-        <v>22.076753616333</v>
+        <v>21.2543029785156</v>
       </c>
       <c r="T15">
-        <v>-1.08323669433594</v>
+        <v>0.0661220550537109</v>
       </c>
       <c r="U15">
-        <v>-0.658237457275391</v>
+        <v>0.0961227416992188</v>
       </c>
       <c r="V15">
-        <v>0.309999465942383</v>
+        <v>0.235000610351563</v>
       </c>
     </row>
     <row r="16" ht="19.5" customHeight="1">
       <c r="A16" s="2">
-        <v>46230</v>
+        <v>46244</v>
       </c>
       <c r="B16">
-        <v>0.0614776611328125</v>
+        <v>-0.10870361328125</v>
       </c>
       <c r="C16">
-        <v>0.492366790771484</v>
+        <v>-0.670436859130859</v>
       </c>
       <c r="D16">
-        <v>0.314016342163086</v>
+        <v>-0.835453033447266</v>
       </c>
       <c r="E16">
-        <v>21.7900009155273</v>
+        <v>20.2399997711182</v>
       </c>
       <c r="F16">
-        <v>22.6501998901367</v>
+        <v>20.2999992370605</v>
       </c>
       <c r="G16">
-        <v>21.7399997711182</v>
+        <v>20.0200004577637</v>
       </c>
       <c r="H16">
-        <v>22.2099990844727</v>
+        <v>20.2099990844727</v>
       </c>
       <c r="I16">
-        <v>21.9311256408691</v>
+        <v>20.5593681335449</v>
       </c>
       <c r="J16">
-        <v>21.6211280822754</v>
+        <v>20.2264862060547</v>
       </c>
       <c r="K16">
-        <v>10710200</v>
+        <v>6569000</v>
       </c>
       <c r="L16">
-        <v>-0.0933333784341812</v>
+        <v>-0.0297619048506021</v>
       </c>
       <c r="M16">
-        <v>30.2797069549561</v>
+        <v>38.257740020752</v>
       </c>
       <c r="N16">
-        <v>-30.4949016571045</v>
+        <v>-0.424057513475418</v>
       </c>
       <c r="O16" t="s">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="P16">
-        <v>-12.2645654678345</v>
+        <v>95.0116653442383</v>
       </c>
       <c r="Q16">
-        <v>22.1088218688965</v>
+        <v>20.4868125915527</v>
       </c>
       <c r="R16">
-        <v>22.2200508117676</v>
+        <v>21.0531120300293</v>
       </c>
       <c r="S16">
-        <v>22.1065673828125</v>
+        <v>21.3902626037598</v>
       </c>
       <c r="T16">
-        <v>-0.719074249267578</v>
+        <v>0.259368896484375</v>
       </c>
       <c r="U16">
-        <v>-0.118871688842773</v>
+        <v>0.206485748291016</v>
       </c>
       <c r="V16">
-        <v>0.30999755859375</v>
+        <v>0.332881927490234</v>
       </c>
     </row>
     <row r="17" ht="19.5" customHeight="1">
       <c r="A17" s="2">
-        <v>46227</v>
+        <v>46241</v>
       </c>
       <c r="B17">
-        <v>0.364728927612305</v>
+        <v>-0.14726448059082</v>
       </c>
       <c r="C17">
-        <v>0.523643493652344</v>
+        <v>-0.642946243286133</v>
       </c>
       <c r="D17">
-        <v>0.401021957397461</v>
+        <v>-0.803007125854492</v>
       </c>
       <c r="E17">
-        <v>22.5200004577637</v>
+        <v>20.2600002288818</v>
       </c>
       <c r="F17">
-        <v>22.6100006103516</v>
+        <v>20.4150009155273</v>
       </c>
       <c r="G17">
-        <v>21.8150005340576</v>
+        <v>20.1800003051758</v>
       </c>
       <c r="H17">
-        <v>22.3600006103516</v>
+        <v>20.3199996948242</v>
       </c>
       <c r="I17">
-        <v>22.3410835266113</v>
+        <v>20.7853908538818</v>
       </c>
       <c r="J17">
-        <v>22.0310840606689</v>
+        <v>20.0895118713379</v>
       </c>
       <c r="K17">
-        <v>9033100</v>
+        <v>6660500</v>
       </c>
       <c r="L17">
-        <v>-0.0938094928860664</v>
+        <v>-0.0459523871541023</v>
       </c>
       <c r="M17">
-        <v>43.5647277832031</v>
+        <v>38.4206657409668</v>
       </c>
       <c r="N17">
-        <v>-4.82013702392578</v>
+        <v>-10.2513265609741</v>
       </c>
       <c r="O17" t="s">
         <v>1</v>
       </c>
       <c r="P17">
-        <v>62.8155326843262</v>
+        <v>15.8023986816406</v>
       </c>
       <c r="Q17">
-        <v>22.2962551116943</v>
+        <v>20.6419906616211</v>
       </c>
       <c r="R17">
-        <v>22.1840209960938</v>
+        <v>21.3021640777588</v>
       </c>
       <c r="S17">
-        <v>22.1268882751465</v>
+        <v>21.527416229248</v>
       </c>
       <c r="T17">
-        <v>-0.268917083740234</v>
+        <v>0.370389938354492</v>
       </c>
       <c r="U17">
-        <v>0.216083526611328</v>
+        <v>-0.0904884338378906</v>
       </c>
       <c r="V17">
-        <v>0.309999465942383</v>
+        <v>0.695878982543945</v>
       </c>
     </row>
     <row r="18" ht="19.5" customHeight="1">
       <c r="A18" s="2">
-        <v>46226</v>
+        <v>46240</v>
       </c>
       <c r="B18">
-        <v>0.550363540649414</v>
+        <v>-0.0613174438476563</v>
       </c>
       <c r="C18">
-        <v>0.789548873901367</v>
+        <v>-0.548988342285156</v>
       </c>
       <c r="D18">
-        <v>0.471246719360352</v>
+        <v>-0.691572189331055</v>
       </c>
       <c r="E18">
-        <v>22.7399997711182</v>
+        <v>20.7000007629395</v>
       </c>
       <c r="F18">
-        <v>23.1849994659424</v>
+        <v>20.7399997711182</v>
       </c>
       <c r="G18">
-        <v>22.4400005340576</v>
+        <v>20.2049999237061</v>
       </c>
       <c r="H18">
-        <v>22.5200004577637</v>
+        <v>20.2299995422363</v>
       </c>
       <c r="I18">
-        <v>24.120454788208</v>
+        <v>21.2324962615967</v>
       </c>
       <c r="J18">
-        <v>22.4487934112549</v>
+        <v>20.8165054321289</v>
       </c>
       <c r="K18">
-        <v>9946700</v>
+        <v>5901700</v>
       </c>
       <c r="L18">
-        <v>-0.0859523043036461</v>
+        <v>-0.0621428713202477</v>
       </c>
       <c r="M18">
-        <v>45.7709503173828</v>
+        <v>42.8091735839844</v>
       </c>
       <c r="N18">
-        <v>-1.97550892829895</v>
+        <v>48.3031349182129</v>
       </c>
       <c r="O18" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="P18">
-        <v>100</v>
+        <v>-4.02017259597778</v>
       </c>
       <c r="Q18">
-        <v>22.3484687805176</v>
+        <v>20.8864498138428</v>
       </c>
       <c r="R18">
-        <v>22.1976013183594</v>
+        <v>21.5750007629395</v>
       </c>
       <c r="S18">
-        <v>22.1373519897461</v>
+        <v>21.6811447143555</v>
       </c>
       <c r="T18">
-        <v>0.935455322265625</v>
+        <v>0.492496490478516</v>
       </c>
       <c r="U18">
-        <v>0.00879287719726563</v>
+        <v>0.611505508422852</v>
       </c>
       <c r="V18">
-        <v>1.67166137695313</v>
+        <v>0.415990829467773</v>
       </c>
     </row>
     <row r="19" ht="19.5" customHeight="1">
       <c r="A19" s="2">
-        <v>46225</v>
+        <v>46239</v>
       </c>
       <c r="B19">
-        <v>-0.178298950195313</v>
+        <v>-0.285120010375977</v>
       </c>
       <c r="C19">
-        <v>0.268390655517578</v>
+        <v>-0.137289047241211</v>
       </c>
       <c r="D19">
-        <v>0.0192470550537109</v>
+        <v>-0.377473831176758</v>
       </c>
       <c r="E19">
-        <v>21.6000003814697</v>
+        <v>21.3400001525879</v>
       </c>
       <c r="F19">
-        <v>21.8050003051758</v>
+        <v>21.4400005340576</v>
       </c>
       <c r="G19">
-        <v>21.4200000762939</v>
+        <v>20.3799991607666</v>
       </c>
       <c r="H19">
-        <v>21.5499992370605</v>
+        <v>20.5100002288818</v>
       </c>
       <c r="I19">
-        <v>21.9597797393799</v>
+        <v>21.4269924163818</v>
       </c>
       <c r="J19">
-        <v>21.2283191680908</v>
+        <v>20.5687198638916</v>
       </c>
       <c r="K19">
-        <v>5676100</v>
+        <v>11253400</v>
       </c>
       <c r="L19">
-        <v>-0.0730951428413391</v>
+        <v>-0.0469047017395496</v>
       </c>
       <c r="M19">
-        <v>46.6933822631836</v>
+        <v>28.8659934997559</v>
       </c>
       <c r="N19">
-        <v>1.694260597229</v>
+        <v>38.9394416809082</v>
       </c>
       <c r="O19" t="s">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="P19">
-        <v>-12.6038360595703</v>
+        <v>99.9001083374023</v>
       </c>
       <c r="Q19">
-        <v>21.6679534912109</v>
+        <v>21.0118141174316</v>
       </c>
       <c r="R19">
-        <v>21.8605117797852</v>
+        <v>21.9915046691895</v>
       </c>
       <c r="S19">
-        <v>21.9972724914551</v>
+        <v>21.8754062652588</v>
       </c>
       <c r="T19">
-        <v>0.154779434204102</v>
+        <v>-0.0130081176757813</v>
       </c>
       <c r="U19">
-        <v>-0.191680908203125</v>
+        <v>0.188720703125</v>
       </c>
       <c r="V19">
-        <v>0.731460571289063</v>
+        <v>0.858272552490234</v>
       </c>
     </row>
     <row r="20" ht="19.5" customHeight="1">
       <c r="A20" s="2">
-        <v>46224</v>
+        <v>46238</v>
       </c>
       <c r="B20">
-        <v>0.0340709686279297</v>
+        <v>-0.735685348510742</v>
       </c>
       <c r="C20">
-        <v>0.427610397338867</v>
+        <v>0.0724983215332031</v>
       </c>
       <c r="D20">
-        <v>0.116727828979492</v>
+        <v>-0.173707962036133</v>
       </c>
       <c r="E20">
-        <v>21.6399993896484</v>
+        <v>20.7700004577637</v>
       </c>
       <c r="F20">
-        <v>21.9300003051758</v>
+        <v>21.2700004577637</v>
       </c>
       <c r="G20">
+        <v>20.7696990966797</v>
+      </c>
+      <c r="H20">
         <v>21.2700004577637</v>
       </c>
-      <c r="H20">
-        <v>21.3700008392334</v>
-      </c>
       <c r="I20">
-        <v>22.038875579834</v>
+        <v>21.6324405670166</v>
       </c>
       <c r="J20">
-        <v>21.0765724182129</v>
+        <v>19.8532638549805</v>
       </c>
       <c r="K20">
-        <v>5551200</v>
+        <v>7316800</v>
       </c>
       <c r="L20">
-        <v>-0.0583331696689129</v>
+        <v>0.00214295159094036</v>
       </c>
       <c r="M20">
-        <v>45.915454864502</v>
+        <v>20.7759532928467</v>
       </c>
       <c r="N20">
-        <v>7.8785138130188</v>
+        <v>-12.7948808670044</v>
       </c>
       <c r="O20" t="s">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="P20">
-        <v>-0.744179964065552</v>
+        <v>49.2009391784668</v>
       </c>
       <c r="Q20">
-        <v>21.7559871673584</v>
+        <v>21.1883125305176</v>
       </c>
       <c r="R20">
-        <v>21.9554901123047</v>
+        <v>22.2094955444336</v>
       </c>
       <c r="S20">
-        <v>22.0733184814453</v>
+        <v>21.9951305389404</v>
       </c>
       <c r="T20">
-        <v>0.108875274658203</v>
+        <v>0.36244010925293</v>
       </c>
       <c r="U20">
-        <v>-0.193428039550781</v>
+        <v>-0.916435241699219</v>
       </c>
       <c r="V20">
-        <v>0.962303161621094</v>
+        <v>1.77917671203613</v>
       </c>
     </row>
     <row r="21" ht="19.5" customHeight="1">
       <c r="A21" s="2">
-        <v>46223</v>
+        <v>46237</v>
       </c>
       <c r="B21">
-        <v>0.391925811767578</v>
+        <v>-0.65983772277832</v>
       </c>
       <c r="C21">
-        <v>0.492935180664063</v>
+        <v>0.0400638580322266</v>
       </c>
       <c r="D21">
-        <v>0.152450561523438</v>
+        <v>-0.0176563262939453</v>
       </c>
       <c r="E21">
-        <v>21.7000007629395</v>
+        <v>21.0699996948242</v>
       </c>
       <c r="F21">
-        <v>22.2549991607666</v>
+        <v>21.1800003051758</v>
       </c>
       <c r="G21">
-        <v>21.4500007629395</v>
+        <v>20.8950004577637</v>
       </c>
       <c r="H21">
-        <v>22.1200008392334</v>
+        <v>21.0799999237061</v>
       </c>
       <c r="I21">
-        <v>22.4566345214844</v>
+        <v>21.4725818634033</v>
       </c>
       <c r="J21">
-        <v>21.430871963501</v>
+        <v>20.4887065887451</v>
       </c>
       <c r="K21">
-        <v>6942700</v>
+        <v>6825100</v>
       </c>
       <c r="L21">
-        <v>-0.042142778635025</v>
+        <v>-0.0326189324259758</v>
       </c>
       <c r="M21">
-        <v>42.5621871948242</v>
+        <v>23.8242359161377</v>
       </c>
       <c r="N21">
-        <v>-25.350830078125</v>
+        <v>-17.6793479919434</v>
       </c>
       <c r="O21" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="P21">
-        <v>3.66390585899353</v>
+        <v>-61.7687721252441</v>
       </c>
       <c r="Q21">
-        <v>22.0166187286377</v>
+        <v>21.4585494995117</v>
       </c>
       <c r="R21">
-        <v>21.960412979126</v>
+        <v>22.2541065216064</v>
       </c>
       <c r="S21">
-        <v>22.133544921875</v>
+        <v>22.0823230743408</v>
       </c>
       <c r="T21">
-        <v>0.201635360717773</v>
+        <v>0.292581558227539</v>
       </c>
       <c r="U21">
-        <v>-0.0191287994384766</v>
+        <v>-0.406293869018555</v>
       </c>
       <c r="V21">
-        <v>1.0257625579834</v>
+        <v>0.983875274658203</v>
       </c>
     </row>
     <row r="22" ht="19.5" customHeight="1">
       <c r="A22" s="2">
-        <v>46220</v>
+        <v>46234</v>
       </c>
       <c r="B22">
-        <v>0.603134155273438</v>
+        <v>-0.393699645996094</v>
       </c>
       <c r="C22">
-        <v>0.456741333007813</v>
+        <v>0.704631805419922</v>
       </c>
       <c r="D22">
-        <v>-0.0313358306884766</v>
+        <v>0.512554168701172</v>
       </c>
       <c r="E22">
-        <v>22.7600002288818</v>
+        <v>21.6399993896484</v>
       </c>
       <c r="F22">
-        <v>22.8400001525879</v>
+        <v>22.5100002288818</v>
       </c>
       <c r="G22">
-        <v>22.0599994659424</v>
+        <v>21.1800003051758</v>
       </c>
       <c r="H22">
-        <v>22.4799995422363</v>
+        <v>21.25</v>
       </c>
       <c r="I22">
-        <v>22.914737701416</v>
+        <v>22.9274063110352</v>
       </c>
       <c r="J22">
-        <v>22.4017143249512</v>
+        <v>20.3054065704346</v>
       </c>
       <c r="K22">
-        <v>10089400</v>
+        <v>8503300</v>
       </c>
       <c r="L22">
-        <v>-0.0073808035813272</v>
+        <v>-0.0340474434196949</v>
       </c>
       <c r="M22">
-        <v>57.0162887573242</v>
+        <v>28.9407768249512</v>
       </c>
       <c r="N22">
-        <v>-1.97543406486511</v>
+        <v>28.6269283294678</v>
       </c>
       <c r="O22" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="P22">
-        <v>95.455940246582</v>
+        <v>-22.4164390563965</v>
       </c>
       <c r="Q22">
-        <v>22.0313625335693</v>
+        <v>21.9039173126221</v>
       </c>
       <c r="R22">
-        <v>21.8592166900635</v>
+        <v>22.6548538208008</v>
       </c>
       <c r="S22">
-        <v>22.1243572235107</v>
+        <v>22.2817363739014</v>
       </c>
       <c r="T22">
-        <v>0.074737548828125</v>
+        <v>0.41740608215332</v>
       </c>
       <c r="U22">
-        <v>0.341714859008789</v>
+        <v>-0.874593734741211</v>
       </c>
       <c r="V22">
-        <v>0.513023376464844</v>
+        <v>2.62199974060059</v>
       </c>
     </row>
     <row r="23" ht="19.5" customHeight="1">
       <c r="A23" s="2">
-        <v>46219</v>
+        <v>46233</v>
       </c>
       <c r="B23">
-        <v>0.109506607055664</v>
+        <v>-0.0996761322021484</v>
       </c>
       <c r="C23">
-        <v>-0.201303482055664</v>
+        <v>1.02289772033691</v>
       </c>
       <c r="D23">
-        <v>-0.543678283691406</v>
+        <v>0.774198532104492</v>
       </c>
       <c r="E23">
-        <v>21.1599998474121</v>
+        <v>22.4799995422363</v>
       </c>
       <c r="F23">
-        <v>21.6749992370605</v>
+        <v>22.7700004577637</v>
       </c>
       <c r="G23">
-        <v>20.9412994384766</v>
+        <v>21.8199996948242</v>
       </c>
       <c r="H23">
-        <v>21.4500007629395</v>
+        <v>21.8199996948242</v>
       </c>
       <c r="I23">
-        <v>21.7233467102051</v>
+        <v>23.2930679321289</v>
       </c>
       <c r="J23">
-        <v>21.4133491516113</v>
+        <v>20.6710681915283</v>
       </c>
       <c r="K23">
-        <v>7337300</v>
+        <v>9302900</v>
       </c>
       <c r="L23">
-        <v>0.00785727705806494</v>
+        <v>-0.0169046483933926</v>
       </c>
       <c r="M23">
-        <v>58.1653060913086</v>
+        <v>22.4997806549072</v>
       </c>
       <c r="N23">
-        <v>-17.4168739318848</v>
+        <v>300.6494140625</v>
       </c>
       <c r="O23" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="P23">
-        <v>-7.64209318161011</v>
+        <v>-31.0044631958008</v>
       </c>
       <c r="Q23">
-        <v>21.4642848968506</v>
+        <v>22.3125190734863</v>
       </c>
       <c r="R23">
-        <v>21.5118846893311</v>
+        <v>22.8138961791992</v>
       </c>
       <c r="S23">
-        <v>22.021390914917</v>
+        <v>22.3450241088867</v>
       </c>
       <c r="T23">
-        <v>0.0483474731445313</v>
+        <v>0.523067474365234</v>
       </c>
       <c r="U23">
-        <v>0.472049713134766</v>
+        <v>-1.1489315032959</v>
       </c>
       <c r="V23">
-        <v>0.30999755859375</v>
+        <v>2.62199974060059</v>
       </c>
     </row>
     <row r="24" ht="19.5" customHeight="1">
       <c r="A24" s="2">
-        <v>46218</v>
+        <v>46232</v>
       </c>
       <c r="B24">
-        <v>-0.0673770904541016</v>
+        <v>0.441112518310547</v>
       </c>
       <c r="C24">
-        <v>-0.317070007324219</v>
+        <v>0.785587310791016</v>
       </c>
       <c r="D24">
-        <v>-0.687747955322266</v>
+        <v>0.695182800292969</v>
       </c>
       <c r="E24">
-        <v>21.2099990844727</v>
+        <v>22.3500003814697</v>
       </c>
       <c r="F24">
-        <v>21.4799995422363</v>
+        <v>23.5100002288818</v>
       </c>
       <c r="G24">
-        <v>20.8299999237061</v>
+        <v>21.7950000762939</v>
       </c>
       <c r="H24">
-        <v>20.8500003814697</v>
+        <v>23.4200000762939</v>
       </c>
       <c r="I24">
-        <v>21.3572006225586</v>
+        <v>24.9417915344238</v>
       </c>
       <c r="J24">
-        <v>21.0471992492676</v>
+        <v>22.3197937011719</v>
       </c>
       <c r="K24">
-        <v>5730800</v>
+        <v>18832500</v>
       </c>
       <c r="L24">
-        <v>-0.0297618135809898</v>
+        <v>-0.00976181030273438</v>
       </c>
       <c r="M24">
-        <v>70.4324340820313</v>
+        <v>5.61582803726196</v>
       </c>
       <c r="N24">
-        <v>21.2787456512451</v>
+        <v>-80.1277160644531</v>
       </c>
       <c r="O24" t="s">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="P24">
-        <v>-23.9522762298584</v>
+        <v>64.2163772583008</v>
       </c>
       <c r="Q24">
-        <v>21.3994331359863</v>
+        <v>22.6965599060059</v>
       </c>
       <c r="R24">
-        <v>21.5538291931152</v>
+        <v>22.5893497467041</v>
       </c>
       <c r="S24">
-        <v>22.0920276641846</v>
+        <v>22.2805633544922</v>
       </c>
       <c r="T24">
-        <v>-0.122798919677734</v>
+        <v>1.43179130554199</v>
       </c>
       <c r="U24">
-        <v>0.217199325561523</v>
+        <v>0.52479362487793</v>
       </c>
       <c r="V24">
-        <v>0.310001373291016</v>
+        <v>2.62199783325195</v>
       </c>
     </row>
     <row r="25" ht="19.5" customHeight="1">
       <c r="A25" s="2">
-        <v>46217</v>
+        <v>46231</v>
       </c>
       <c r="B25">
-        <v>0.136562347412109</v>
+        <v>-0.407449722290039</v>
       </c>
       <c r="C25">
-        <v>-0.232601165771484</v>
+        <v>0.318998336791992</v>
       </c>
       <c r="D25">
-        <v>-0.703542709350586</v>
+        <v>0.211315155029297</v>
       </c>
       <c r="E25">
-        <v>21.4400005340576</v>
+        <v>22.1949996948242</v>
       </c>
       <c r="F25">
-        <v>21.6100006103516</v>
+        <v>22.5599994659424</v>
       </c>
       <c r="G25">
-        <v>21.2299995422363</v>
+        <v>21.8250007629395</v>
       </c>
       <c r="H25">
-        <v>21.5100002288818</v>
+        <v>22.0300006866455</v>
       </c>
       <c r="I25">
-        <v>22.0717163085938</v>
+        <v>21.4767627716064</v>
       </c>
       <c r="J25">
-        <v>21.5998001098633</v>
+        <v>21.1667633056641</v>
       </c>
       <c r="K25">
-        <v>4459700</v>
+        <v>6852400</v>
       </c>
       <c r="L25">
-        <v>-0.0488094165921211</v>
+        <v>-0.0754761472344398</v>
       </c>
       <c r="M25">
-        <v>58.074836730957</v>
+        <v>28.2595958709717</v>
       </c>
       <c r="N25">
-        <v>-0.175840109586716</v>
+        <v>-6.67150163650513</v>
       </c>
       <c r="O25" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="P25">
-        <v>7.82178258895874</v>
+        <v>-20.5401268005371</v>
       </c>
       <c r="Q25">
-        <v>21.7143611907959</v>
+        <v>21.8332195281982</v>
       </c>
       <c r="R25">
-        <v>21.7141742706299</v>
+        <v>22.1766109466553</v>
       </c>
       <c r="S25">
-        <v>22.2298221588135</v>
+        <v>22.076753616333</v>
       </c>
       <c r="T25">
-        <v>0.461715698242188</v>
+        <v>-1.08323669433594</v>
       </c>
       <c r="U25">
-        <v>0.369800567626953</v>
+        <v>-0.658237457275391</v>
       </c>
       <c r="V25">
-        <v>0.471916198730469</v>
+        <v>0.309999465942383</v>
       </c>
     </row>
     <row r="26" ht="19.5" customHeight="1">
       <c r="A26" s="2">
-        <v>46216</v>
+        <v>46230</v>
       </c>
       <c r="B26">
-        <v>0.12352180480957</v>
+        <v>0.0614776611328125</v>
       </c>
       <c r="C26">
-        <v>-0.299781799316406</v>
+        <v>0.492366790771484</v>
       </c>
       <c r="D26">
-        <v>-0.722906112670898</v>
+        <v>0.314016342163086</v>
       </c>
       <c r="E26">
-        <v>21.3600006103516</v>
+        <v>21.7900009155273</v>
       </c>
       <c r="F26">
-        <v>21.9599990844727</v>
+        <v>22.6501998901367</v>
       </c>
       <c r="G26">
-        <v>21.1299991607666</v>
+        <v>21.7399997711182</v>
       </c>
       <c r="H26">
-        <v>21.7800006866455</v>
+        <v>22.2099990844727</v>
       </c>
       <c r="I26">
-        <v>22.1969223022461</v>
+        <v>21.9311256408691</v>
       </c>
       <c r="J26">
-        <v>21.8869247436523</v>
+        <v>21.6211280822754</v>
       </c>
       <c r="K26">
-        <v>8190000</v>
+        <v>10710200</v>
       </c>
       <c r="L26">
-        <v>-0.105952307581902</v>
+        <v>-0.0933333784341812</v>
       </c>
       <c r="M26">
-        <v>58.1771354675293</v>
+        <v>30.2797069549561</v>
       </c>
       <c r="N26">
-        <v>-5.97548294067383</v>
+        <v>-30.4949016571045</v>
       </c>
       <c r="O26" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="P26">
-        <v>0.707083880901337</v>
+        <v>-12.2645654678345</v>
       </c>
       <c r="Q26">
-        <v>21.7029037475586</v>
+        <v>22.1088218688965</v>
       </c>
       <c r="R26">
-        <v>21.7794609069824</v>
+        <v>22.2200508117676</v>
       </c>
       <c r="S26">
-        <v>22.3239288330078</v>
+        <v>22.1065673828125</v>
       </c>
       <c r="T26">
-        <v>0.236923217773438</v>
+        <v>-0.719074249267578</v>
       </c>
       <c r="U26">
-        <v>0.756925582885742</v>
+        <v>-0.118871688842773</v>
       </c>
       <c r="V26">
         <v>0.30999755859375</v>
@@ -2199,1226 +2199,1294 @@
     </row>
     <row r="27" ht="19.5" customHeight="1">
       <c r="A27" s="2">
-        <v>46213</v>
+        <v>46227</v>
       </c>
       <c r="B27">
-        <v>-0.204776763916016</v>
+        <v>0.364728927612305</v>
       </c>
       <c r="C27">
-        <v>-0.347467422485352</v>
+        <v>0.523643493652344</v>
       </c>
       <c r="D27">
-        <v>-0.727428436279297</v>
+        <v>0.401021957397461</v>
       </c>
       <c r="E27">
-        <v>21.5</v>
+        <v>22.5200004577637</v>
       </c>
       <c r="F27">
-        <v>22.0200004577637</v>
+        <v>22.6100006103516</v>
       </c>
       <c r="G27">
-        <v>21.0650005340576</v>
+        <v>21.8150005340576</v>
       </c>
       <c r="H27">
-        <v>21.1299991607666</v>
+        <v>22.3600006103516</v>
       </c>
       <c r="I27">
-        <v>22.118709564209</v>
+        <v>22.3410835266113</v>
       </c>
       <c r="J27">
-        <v>20.6618118286133</v>
+        <v>22.0310840606689</v>
       </c>
       <c r="K27">
-        <v>5787900</v>
+        <v>9033100</v>
       </c>
       <c r="L27">
-        <v>-0.0845237001776695</v>
+        <v>-0.0938094928860664</v>
       </c>
       <c r="M27">
-        <v>61.8744316101074</v>
+        <v>43.5647277832031</v>
       </c>
       <c r="N27">
-        <v>15.8251628875732</v>
+        <v>-4.82013702392578</v>
       </c>
       <c r="O27" t="s">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="P27">
-        <v>-0.00522141391411424</v>
+        <v>62.8155326843262</v>
       </c>
       <c r="Q27">
-        <v>21.4506454467773</v>
+        <v>22.2962551116943</v>
       </c>
       <c r="R27">
-        <v>21.8880519866943</v>
+        <v>22.1840209960938</v>
       </c>
       <c r="S27">
-        <v>22.4147987365723</v>
+        <v>22.1268882751465</v>
       </c>
       <c r="T27">
-        <v>0.0987091064453125</v>
+        <v>-0.268917083740234</v>
       </c>
       <c r="U27">
-        <v>-0.403188705444336</v>
+        <v>0.216083526611328</v>
       </c>
       <c r="V27">
-        <v>1.4568977355957</v>
+        <v>0.309999465942383</v>
       </c>
     </row>
     <row r="28" ht="19.5" customHeight="1">
       <c r="A28" s="2">
-        <v>46212</v>
+        <v>46226</v>
       </c>
       <c r="B28">
-        <v>-0.243209838867188</v>
+        <v>0.550363540649414</v>
       </c>
       <c r="C28">
-        <v>-0.204446792602539</v>
+        <v>0.789548873901367</v>
       </c>
       <c r="D28">
-        <v>-0.655893325805664</v>
+        <v>0.471246719360352</v>
       </c>
       <c r="E28">
-        <v>21.8600006103516</v>
+        <v>22.7399997711182</v>
       </c>
       <c r="F28">
-        <v>22.1000003814697</v>
+        <v>23.1849994659424</v>
       </c>
       <c r="G28">
-        <v>21.5799999237061</v>
+        <v>22.4400005340576</v>
       </c>
       <c r="H28">
-        <v>21.5799999237061</v>
+        <v>22.5200004577637</v>
       </c>
       <c r="I28">
-        <v>22.3199882507324</v>
+        <v>24.120454788208</v>
       </c>
       <c r="J28">
-        <v>20.0562515258789</v>
+        <v>22.4487934112549</v>
       </c>
       <c r="K28">
-        <v>4864800</v>
+        <v>9946700</v>
       </c>
       <c r="L28">
-        <v>-0.0345236472785473</v>
+        <v>-0.0859523043036461</v>
       </c>
       <c r="M28">
-        <v>53.4205436706543</v>
+        <v>45.7709503173828</v>
       </c>
       <c r="N28">
-        <v>10.6338014602661</v>
+        <v>-1.97550892829895</v>
       </c>
       <c r="O28" t="s">
         <v>1</v>
       </c>
       <c r="P28">
-        <v>29.9308681488037</v>
+        <v>100</v>
       </c>
       <c r="Q28">
-        <v>21.5979118347168</v>
+        <v>22.3484687805176</v>
       </c>
       <c r="R28">
-        <v>22.1009502410889</v>
+        <v>22.1976013183594</v>
       </c>
       <c r="S28">
-        <v>22.5637645721436</v>
+        <v>22.1373519897461</v>
       </c>
       <c r="T28">
-        <v>0.219987869262695</v>
+        <v>0.935455322265625</v>
       </c>
       <c r="U28">
-        <v>-1.52374839782715</v>
+        <v>0.00879287719726563</v>
       </c>
       <c r="V28">
-        <v>2.26373672485352</v>
+        <v>1.67166137695313</v>
       </c>
     </row>
     <row r="29" ht="19.5" customHeight="1">
       <c r="A29" s="2">
-        <v>46211</v>
+        <v>46225</v>
       </c>
       <c r="B29">
-        <v>0.00951385498046875</v>
+        <v>-0.178298950195313</v>
       </c>
       <c r="C29">
-        <v>-0.355205535888672</v>
+        <v>0.268390655517578</v>
       </c>
       <c r="D29">
-        <v>-0.625932693481445</v>
+        <v>0.0192470550537109</v>
       </c>
       <c r="E29">
-        <v>22.1599998474121</v>
+        <v>21.6000003814697</v>
       </c>
       <c r="F29">
-        <v>22.7900009155273</v>
+        <v>21.8050003051758</v>
       </c>
       <c r="G29">
-        <v>21.7299995422363</v>
+        <v>21.4200000762939</v>
       </c>
       <c r="H29">
-        <v>22.0100002288818</v>
+        <v>21.5499992370605</v>
       </c>
       <c r="I29">
-        <v>23.8744087219238</v>
+        <v>21.9597797393799</v>
       </c>
       <c r="J29">
-        <v>20.4272975921631</v>
+        <v>21.2283191680908</v>
       </c>
       <c r="K29">
-        <v>8076200</v>
+        <v>5676100</v>
       </c>
       <c r="L29">
-        <v>-0.0145236421376467</v>
+        <v>-0.0730951428413391</v>
       </c>
       <c r="M29">
-        <v>48.2859153747559</v>
+        <v>46.6933822631836</v>
       </c>
       <c r="N29">
-        <v>54.1862564086914</v>
+        <v>1.694260597229</v>
       </c>
       <c r="O29" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="P29">
-        <v>-4.73143672943115</v>
+        <v>-12.6038360595703</v>
       </c>
       <c r="Q29">
-        <v>21.8777961730957</v>
+        <v>21.6679534912109</v>
       </c>
       <c r="R29">
-        <v>22.1314544677734</v>
+        <v>21.8605117797852</v>
       </c>
       <c r="S29">
-        <v>22.6682186126709</v>
+        <v>21.9972724914551</v>
       </c>
       <c r="T29">
-        <v>1.08440780639648</v>
+        <v>0.154779434204102</v>
       </c>
       <c r="U29">
-        <v>-1.30270195007324</v>
+        <v>-0.191680908203125</v>
       </c>
       <c r="V29">
-        <v>3.44711112976074</v>
+        <v>0.731460571289063</v>
       </c>
     </row>
     <row r="30" ht="19.5" customHeight="1">
       <c r="A30" s="2">
-        <v>46210</v>
+        <v>46224</v>
       </c>
       <c r="B30">
-        <v>-0.375518798828125</v>
+        <v>0.0340709686279297</v>
       </c>
       <c r="C30">
-        <v>-1.15375328063965</v>
+        <v>0.427610397338867</v>
       </c>
       <c r="D30">
-        <v>-1.03360176086426</v>
+        <v>0.116727828979492</v>
       </c>
       <c r="E30">
-        <v>21.4899997711182</v>
+        <v>21.6399993896484</v>
       </c>
       <c r="F30">
-        <v>21.9549999237061</v>
+        <v>21.9300003051758</v>
       </c>
       <c r="G30">
-        <v>21.3250007629395</v>
+        <v>21.2700004577637</v>
       </c>
       <c r="H30">
-        <v>21.6900005340576</v>
+        <v>21.3700008392334</v>
       </c>
       <c r="I30">
-        <v>21.8200778961182</v>
+        <v>22.038875579834</v>
       </c>
       <c r="J30">
-        <v>21.0972957611084</v>
+        <v>21.0765724182129</v>
       </c>
       <c r="K30">
-        <v>7265900</v>
+        <v>5551200</v>
       </c>
       <c r="L30">
-        <v>0.0607143566012383</v>
+        <v>-0.0583331696689129</v>
       </c>
       <c r="M30">
-        <v>31.316614151001</v>
+        <v>45.915454864502</v>
       </c>
       <c r="N30">
-        <v>-5.85662317276001</v>
+        <v>7.8785138130188</v>
       </c>
       <c r="O30" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="P30">
-        <v>7.77024745941162</v>
+        <v>-0.744179964065552</v>
       </c>
       <c r="Q30">
-        <v>21.6503143310547</v>
+        <v>21.7559871673584</v>
       </c>
       <c r="R30">
-        <v>21.8759937286377</v>
+        <v>21.9554901123047</v>
       </c>
       <c r="S30">
-        <v>22.630199432373</v>
+        <v>22.0733184814453</v>
       </c>
       <c r="T30">
-        <v>-0.134922027587891</v>
+        <v>0.108875274658203</v>
       </c>
       <c r="U30">
-        <v>-0.227705001831055</v>
+        <v>-0.193428039550781</v>
       </c>
       <c r="V30">
-        <v>0.722782135009766</v>
+        <v>0.962303161621094</v>
       </c>
     </row>
     <row r="31" ht="19.5" customHeight="1">
       <c r="A31" s="2">
-        <v>46209</v>
+        <v>46223</v>
       </c>
       <c r="B31">
-        <v>-0.518081665039063</v>
+        <v>0.391925811767578</v>
       </c>
       <c r="C31">
-        <v>-1.2119312286377</v>
+        <v>0.492935180664063</v>
       </c>
       <c r="D31">
-        <v>-1.10026741027832</v>
+        <v>0.152450561523438</v>
       </c>
       <c r="E31">
-        <v>21.7199993133545</v>
+        <v>21.7000007629395</v>
       </c>
       <c r="F31">
-        <v>21.7199993133545</v>
+        <v>22.2549991607666</v>
       </c>
       <c r="G31">
-        <v>21.4099998474121</v>
+        <v>21.4500007629395</v>
       </c>
       <c r="H31">
-        <v>21.4899997711182</v>
+        <v>22.1200008392334</v>
       </c>
       <c r="I31">
-        <v>21.8874111175537</v>
+        <v>22.4566345214844</v>
       </c>
       <c r="J31">
-        <v>20.5938625335693</v>
+        <v>21.430871963501</v>
       </c>
       <c r="K31">
-        <v>6209900</v>
+        <v>6942700</v>
       </c>
       <c r="L31">
-        <v>0.00357146491296589</v>
+        <v>-0.042142778635025</v>
       </c>
       <c r="M31">
-        <v>33.2648086547852</v>
+        <v>42.5621871948242</v>
       </c>
       <c r="N31">
-        <v>-9.78374195098877</v>
+        <v>-25.350830078125</v>
       </c>
       <c r="O31" t="s">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="P31">
-        <v>-13.5685234069824</v>
+        <v>3.66390585899353</v>
       </c>
       <c r="Q31">
-        <v>21.7651062011719</v>
+        <v>22.0166187286377</v>
       </c>
       <c r="R31">
-        <v>21.9957885742188</v>
+        <v>21.960412979126</v>
       </c>
       <c r="S31">
-        <v>22.7744026184082</v>
+        <v>22.133544921875</v>
       </c>
       <c r="T31">
-        <v>0.167411804199219</v>
+        <v>0.201635360717773</v>
       </c>
       <c r="U31">
-        <v>-0.816137313842773</v>
+        <v>-0.0191287994384766</v>
       </c>
       <c r="V31">
-        <v>1.29354858398438</v>
+        <v>1.0257625579834</v>
       </c>
     </row>
     <row r="32" ht="19.5" customHeight="1">
       <c r="A32" s="2">
-        <v>46205</v>
+        <v>46220</v>
       </c>
       <c r="B32">
-        <v>-0.419429779052734</v>
+        <v>0.603134155273438</v>
       </c>
       <c r="C32">
-        <v>-0.915922164916992</v>
+        <v>0.456741333007813</v>
       </c>
       <c r="D32">
-        <v>-1.01813888549805</v>
+        <v>-0.0313358306884766</v>
       </c>
       <c r="E32">
+        <v>22.7600002288818</v>
+      </c>
+      <c r="F32">
+        <v>22.8400001525879</v>
+      </c>
+      <c r="G32">
         <v>22.0599994659424</v>
       </c>
-      <c r="F32">
-        <v>22.5849990844727</v>
-      </c>
-      <c r="G32">
-        <v>21.7350006103516</v>
-      </c>
       <c r="H32">
-        <v>22.0400009155273</v>
+        <v>22.4799995422363</v>
       </c>
       <c r="I32">
-        <v>22.1091861724854</v>
+        <v>22.914737701416</v>
       </c>
       <c r="J32">
-        <v>21.7441864013672</v>
+        <v>22.4017143249512</v>
       </c>
       <c r="K32">
-        <v>9001800</v>
+        <v>10089400</v>
       </c>
       <c r="L32">
-        <v>0.00547617953270674</v>
+        <v>-0.0073808035813272</v>
       </c>
       <c r="M32">
-        <v>36.8722991943359</v>
+        <v>57.0162887573242</v>
       </c>
       <c r="N32">
-        <v>-19.0741996765137</v>
+        <v>-1.97543406486511</v>
       </c>
       <c r="O32" t="s">
         <v>1</v>
       </c>
       <c r="P32">
-        <v>9.51707172393799</v>
+        <v>95.455940246582</v>
       </c>
       <c r="Q32">
-        <v>22.2072486877441</v>
+        <v>22.0313625335693</v>
       </c>
       <c r="R32">
-        <v>22.3150157928467</v>
+        <v>21.8592166900635</v>
       </c>
       <c r="S32">
-        <v>22.9963321685791</v>
+        <v>22.1243572235107</v>
       </c>
       <c r="T32">
-        <v>-0.475812911987305</v>
+        <v>0.074737548828125</v>
       </c>
       <c r="U32">
-        <v>0.009185791015625</v>
+        <v>0.341714859008789</v>
       </c>
       <c r="V32">
-        <v>0.364999771118164</v>
+        <v>0.513023376464844</v>
       </c>
     </row>
     <row r="33" ht="19.5" customHeight="1">
       <c r="A33" s="2">
-        <v>46204</v>
+        <v>46219</v>
       </c>
       <c r="B33">
-        <v>-0.405847549438477</v>
+        <v>0.109506607055664</v>
       </c>
       <c r="C33">
-        <v>-0.976701736450195</v>
+        <v>-0.201303482055664</v>
       </c>
       <c r="D33">
-        <v>-1.17591094970703</v>
+        <v>-0.543678283691406</v>
       </c>
       <c r="E33">
-        <v>22.3500003814697</v>
+        <v>21.1599998474121</v>
       </c>
       <c r="F33">
-        <v>22.5499992370605</v>
+        <v>21.6749992370605</v>
       </c>
       <c r="G33">
-        <v>22.0102996826172</v>
+        <v>20.9412994384766</v>
       </c>
       <c r="H33">
-        <v>22.3199996948242</v>
+        <v>21.4500007629395</v>
       </c>
       <c r="I33">
-        <v>22.6419010162354</v>
+        <v>21.7233467102051</v>
       </c>
       <c r="J33">
-        <v>22.0874977111816</v>
+        <v>21.4133491516113</v>
       </c>
       <c r="K33">
-        <v>7270600</v>
+        <v>7337300</v>
       </c>
       <c r="L33">
-        <v>0.00357137410901487</v>
+        <v>0.00785727705806494</v>
       </c>
       <c r="M33">
-        <v>45.5630950927734</v>
+        <v>58.1653060913086</v>
       </c>
       <c r="N33">
-        <v>-19.3071174621582</v>
+        <v>-17.4168739318848</v>
       </c>
       <c r="O33" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="P33">
-        <v>1.26358222961426</v>
+        <v>-7.64209318161011</v>
       </c>
       <c r="Q33">
-        <v>22.4488906860352</v>
+        <v>21.4642848968506</v>
       </c>
       <c r="R33">
-        <v>22.4495525360107</v>
+        <v>21.5118846893311</v>
       </c>
       <c r="S33">
-        <v>23.1492938995361</v>
+        <v>22.021390914917</v>
       </c>
       <c r="T33">
-        <v>0.0919017791748047</v>
+        <v>0.0483474731445313</v>
       </c>
       <c r="U33">
-        <v>0.0771980285644531</v>
+        <v>0.472049713134766</v>
       </c>
       <c r="V33">
-        <v>0.554403305053711</v>
+        <v>0.30999755859375</v>
       </c>
     </row>
     <row r="34" ht="19.5" customHeight="1">
       <c r="A34" s="2">
-        <v>46203</v>
+        <v>46218</v>
       </c>
       <c r="B34">
-        <v>-0.683012008666992</v>
+        <v>-0.0673770904541016</v>
       </c>
       <c r="C34">
-        <v>-0.766977310180664</v>
+        <v>-0.317070007324219</v>
       </c>
       <c r="D34">
-        <v>-1.12672424316406</v>
+        <v>-0.687747955322266</v>
       </c>
       <c r="E34">
-        <v>22.6000003814697</v>
+        <v>21.2099990844727</v>
       </c>
       <c r="F34">
-        <v>22.7000007629395</v>
+        <v>21.4799995422363</v>
       </c>
       <c r="G34">
-        <v>21.9599990844727</v>
+        <v>20.8299999237061</v>
       </c>
       <c r="H34">
-        <v>22.0900001525879</v>
+        <v>20.8500003814697</v>
       </c>
       <c r="I34">
-        <v>23.2584552764893</v>
+        <v>21.3572006225586</v>
       </c>
       <c r="J34">
-        <v>20.9772338867188</v>
+        <v>21.0471992492676</v>
       </c>
       <c r="K34">
-        <v>4630600</v>
+        <v>5730800</v>
       </c>
       <c r="L34">
-        <v>0.0226190648972988</v>
+        <v>-0.0297618135809898</v>
       </c>
       <c r="M34">
-        <v>56.4648246765137</v>
+        <v>70.4324340820313</v>
       </c>
       <c r="N34">
-        <v>35.7507209777832</v>
+        <v>21.2787456512451</v>
       </c>
       <c r="O34" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="P34">
-        <v>-35.5566825866699</v>
+        <v>-23.9522762298584</v>
       </c>
       <c r="Q34">
-        <v>22.5476150512695</v>
+        <v>21.3994331359863</v>
       </c>
       <c r="R34">
-        <v>22.6672439575195</v>
+        <v>21.5538291931152</v>
       </c>
       <c r="S34">
-        <v>23.3205070495605</v>
+        <v>22.0920276641846</v>
       </c>
       <c r="T34">
-        <v>0.558454513549805</v>
+        <v>-0.122798919677734</v>
       </c>
       <c r="U34">
-        <v>-0.982765197753906</v>
+        <v>0.217199325561523</v>
       </c>
       <c r="V34">
-        <v>2.28122138977051</v>
+        <v>0.310001373291016</v>
       </c>
     </row>
     <row r="35" ht="19.5" customHeight="1">
       <c r="A35" s="2">
-        <v>46202</v>
+        <v>46217</v>
       </c>
       <c r="B35">
-        <v>-0.565788269042969</v>
+        <v>0.136562347412109</v>
       </c>
       <c r="C35">
-        <v>-0.206932067871094</v>
+        <v>-0.232601165771484</v>
       </c>
       <c r="D35">
-        <v>-0.893896102905273</v>
+        <v>-0.703542709350586</v>
       </c>
       <c r="E35">
-        <v>22.8600006103516</v>
+        <v>21.4400005340576</v>
       </c>
       <c r="F35">
-        <v>23.4799995422363</v>
+        <v>21.6100006103516</v>
       </c>
       <c r="G35">
-        <v>22.5149993896484</v>
+        <v>21.2299995422363</v>
       </c>
       <c r="H35">
-        <v>22.5499992370605</v>
+        <v>21.5100002288818</v>
       </c>
       <c r="I35">
-        <v>22.7034931182861</v>
+        <v>22.0717163085938</v>
       </c>
       <c r="J35">
-        <v>21.9739532470703</v>
+        <v>21.5998001098633</v>
       </c>
       <c r="K35">
-        <v>16043900</v>
+        <v>4459700</v>
       </c>
       <c r="L35">
-        <v>0.0426190681755543</v>
+        <v>-0.0488094165921211</v>
       </c>
       <c r="M35">
-        <v>41.5944938659668</v>
+        <v>58.074836730957</v>
       </c>
       <c r="N35">
-        <v>28.7921371459961</v>
+        <v>-0.175840109586716</v>
       </c>
       <c r="O35" t="s">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="P35">
-        <v>-20.1520481109619</v>
+        <v>7.82178258895874</v>
       </c>
       <c r="Q35">
-        <v>22.988452911377</v>
+        <v>21.7143611907959</v>
       </c>
       <c r="R35">
-        <v>23.0405597686768</v>
+        <v>21.7141742706299</v>
       </c>
       <c r="S35">
-        <v>23.5438270568848</v>
+        <v>22.2298221588135</v>
       </c>
       <c r="T35">
-        <v>-0.776506423950195</v>
+        <v>0.461715698242188</v>
       </c>
       <c r="U35">
-        <v>-0.541046142578125</v>
+        <v>0.369800567626953</v>
       </c>
       <c r="V35">
-        <v>0.72953987121582</v>
+        <v>0.471916198730469</v>
       </c>
     </row>
     <row r="36" ht="19.5" customHeight="1">
       <c r="A36" s="2">
-        <v>46199</v>
+        <v>46216</v>
       </c>
       <c r="B36">
-        <v>0.257791519165039</v>
+        <v>0.12352180480957</v>
       </c>
       <c r="C36">
-        <v>0.105573654174805</v>
+        <v>-0.299781799316406</v>
       </c>
       <c r="D36">
-        <v>-0.787239074707031</v>
+        <v>-0.722906112670898</v>
       </c>
       <c r="E36">
-        <v>24.1000003814697</v>
+        <v>21.3600006103516</v>
       </c>
       <c r="F36">
-        <v>24.3299999237061</v>
+        <v>21.9599990844727</v>
       </c>
       <c r="G36">
-        <v>23.2150001525879</v>
+        <v>21.1299991607666</v>
       </c>
       <c r="H36">
-        <v>23.5599994659424</v>
+        <v>21.7800006866455</v>
       </c>
       <c r="I36">
-        <v>24.4937362670898</v>
+        <v>22.1969223022461</v>
       </c>
       <c r="J36">
-        <v>23.3337364196777</v>
+        <v>21.8869247436523</v>
       </c>
       <c r="K36">
-        <v>7342300</v>
+        <v>8190000</v>
       </c>
       <c r="L36">
-        <v>0.0311905089765787</v>
+        <v>-0.105952307581902</v>
       </c>
       <c r="M36">
-        <v>32.2958335876465</v>
+        <v>58.1771354675293</v>
       </c>
       <c r="N36">
-        <v>24.3135643005371</v>
+        <v>-5.97548294067383</v>
       </c>
       <c r="O36" t="s">
         <v>1</v>
       </c>
       <c r="P36">
-        <v>6.54932403564453</v>
+        <v>0.707083880901337</v>
       </c>
       <c r="Q36">
-        <v>23.5688209533691</v>
+        <v>21.7029037475586</v>
       </c>
       <c r="R36">
-        <v>23.2897605895996</v>
+        <v>21.7794609069824</v>
       </c>
       <c r="S36">
-        <v>23.7002143859863</v>
+        <v>22.3239288330078</v>
       </c>
       <c r="T36">
-        <v>0.163736343383789</v>
+        <v>0.236923217773438</v>
       </c>
       <c r="U36">
-        <v>0.118736267089844</v>
+        <v>0.756925582885742</v>
       </c>
       <c r="V36">
-        <v>1.15999984741211</v>
+        <v>0.30999755859375</v>
       </c>
     </row>
     <row r="37" ht="19.5" customHeight="1">
       <c r="A37" s="2">
-        <v>46198</v>
+        <v>46213</v>
       </c>
       <c r="B37">
-        <v>0.0895557403564453</v>
+        <v>-0.204776763916016</v>
       </c>
       <c r="C37">
-        <v>-0.343547821044922</v>
+        <v>-0.347467422485352</v>
       </c>
       <c r="D37">
-        <v>-0.989597320556641</v>
+        <v>-0.727428436279297</v>
       </c>
       <c r="E37">
-        <v>22.8400001525879</v>
+        <v>21.5</v>
       </c>
       <c r="F37">
-        <v>23.7299995422363</v>
+        <v>22.0200004577637</v>
       </c>
       <c r="G37">
-        <v>22.8299999237061</v>
+        <v>21.0650005340576</v>
       </c>
       <c r="H37">
-        <v>23.25</v>
+        <v>21.1299991607666</v>
       </c>
       <c r="I37">
-        <v>23.4458656311035</v>
+        <v>22.118709564209</v>
       </c>
       <c r="J37">
-        <v>23.0127544403076</v>
+        <v>20.6618118286133</v>
       </c>
       <c r="K37">
-        <v>9513800</v>
+        <v>5787900</v>
       </c>
       <c r="L37">
-        <v>0.0383334383368492</v>
+        <v>-0.0845237001776695</v>
       </c>
       <c r="M37">
-        <v>25.9793319702148</v>
+        <v>61.8744316101074</v>
       </c>
       <c r="N37">
-        <v>43.6857986450195</v>
+        <v>15.8251628875732</v>
       </c>
       <c r="O37" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="P37">
-        <v>-4.32447957992554</v>
+        <v>-0.00522141391411424</v>
       </c>
       <c r="Q37">
-        <v>23.3432121276855</v>
+        <v>21.4506454467773</v>
       </c>
       <c r="R37">
-        <v>23.1578369140625</v>
+        <v>21.8880519866943</v>
       </c>
       <c r="S37">
-        <v>23.6892375946045</v>
+        <v>22.4147987365723</v>
       </c>
       <c r="T37">
-        <v>-0.284133911132813</v>
+        <v>0.0987091064453125</v>
       </c>
       <c r="U37">
-        <v>0.182754516601563</v>
+        <v>-0.403188705444336</v>
       </c>
       <c r="V37">
-        <v>0.433111190795898</v>
+        <v>1.4568977355957</v>
       </c>
     </row>
     <row r="38" ht="19.5" customHeight="1">
       <c r="A38" s="2">
-        <v>46197</v>
+        <v>46212</v>
       </c>
       <c r="B38">
-        <v>0.191095352172852</v>
+        <v>-0.243209838867188</v>
       </c>
       <c r="C38">
-        <v>-0.519216537475586</v>
+        <v>-0.204446792602539</v>
       </c>
       <c r="D38">
-        <v>-0.922773361206055</v>
+        <v>-0.655893325805664</v>
       </c>
       <c r="E38">
-        <v>23.6849994659424</v>
+        <v>21.8600006103516</v>
       </c>
       <c r="F38">
-        <v>24.1499996185303</v>
+        <v>22.1000003814697</v>
       </c>
       <c r="G38">
-        <v>23.1499996185303</v>
+        <v>21.5799999237061</v>
       </c>
       <c r="H38">
-        <v>23.6900005340576</v>
+        <v>21.5799999237061</v>
       </c>
       <c r="I38">
-        <v>23.3936557769775</v>
+        <v>22.3199882507324</v>
       </c>
       <c r="J38">
-        <v>23.0286560058594</v>
+        <v>20.0562515258789</v>
       </c>
       <c r="K38">
-        <v>7918300</v>
+        <v>4864800</v>
       </c>
       <c r="L38">
-        <v>0.0133334565907717</v>
+        <v>-0.0345236472785473</v>
       </c>
       <c r="M38">
-        <v>18.0806541442871</v>
+        <v>53.4205436706543</v>
       </c>
       <c r="N38">
-        <v>-32.3323097229004</v>
+        <v>10.6338014602661</v>
       </c>
       <c r="O38" t="s">
         <v>1</v>
       </c>
       <c r="P38">
-        <v>35.4040069580078</v>
+        <v>29.9308681488037</v>
       </c>
       <c r="Q38">
-        <v>23.4488410949707</v>
+        <v>21.5979118347168</v>
       </c>
       <c r="R38">
-        <v>23.2470588684082</v>
+        <v>22.1009502410889</v>
       </c>
       <c r="S38">
-        <v>23.8238086700439</v>
+        <v>22.5637645721436</v>
       </c>
       <c r="T38">
-        <v>-0.756343841552734</v>
+        <v>0.219987869262695</v>
       </c>
       <c r="U38">
-        <v>-0.121343612670898</v>
+        <v>-1.52374839782715</v>
       </c>
       <c r="V38">
-        <v>0.364999771118164</v>
+        <v>2.26373672485352</v>
       </c>
     </row>
     <row r="39" ht="19.5" customHeight="1">
       <c r="A39" s="2">
-        <v>46196</v>
+        <v>46211</v>
       </c>
       <c r="B39">
-        <v>0.624240875244141</v>
+        <v>0.00951385498046875</v>
       </c>
       <c r="C39">
-        <v>-0.840803146362305</v>
+        <v>-0.355205535888672</v>
       </c>
       <c r="D39">
-        <v>-1.08876419067383</v>
+        <v>-0.625932693481445</v>
       </c>
       <c r="E39">
-        <v>23.8199996948242</v>
+        <v>22.1599998474121</v>
       </c>
       <c r="F39">
-        <v>24.1049995422363</v>
+        <v>22.7900009155273</v>
       </c>
       <c r="G39">
-        <v>23.3649997711182</v>
+        <v>21.7299995422363</v>
       </c>
       <c r="H39">
-        <v>23.8700008392334</v>
+        <v>22.0100002288818</v>
       </c>
       <c r="I39">
-        <v>24.4070243835449</v>
+        <v>23.8744087219238</v>
       </c>
       <c r="J39">
-        <v>24.0420265197754</v>
+        <v>20.4272975921631</v>
       </c>
       <c r="K39">
-        <v>10784900</v>
+        <v>8076200</v>
       </c>
       <c r="L39">
-        <v>0.018809637054801</v>
+        <v>-0.0145236421376467</v>
       </c>
       <c r="M39">
-        <v>26.7197742462158</v>
+        <v>48.2859153747559</v>
       </c>
       <c r="N39">
-        <v>-5.11963653564453</v>
+        <v>54.1862564086914</v>
       </c>
       <c r="O39" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="P39">
-        <v>51.3034210205078</v>
+        <v>-4.73143672943115</v>
       </c>
       <c r="Q39">
-        <v>23.5263481140137</v>
+        <v>21.8777961730957</v>
       </c>
       <c r="R39">
-        <v>23.176887512207</v>
+        <v>22.1314544677734</v>
       </c>
       <c r="S39">
-        <v>23.8667259216309</v>
+        <v>22.6682186126709</v>
       </c>
       <c r="T39">
-        <v>0.302024841308594</v>
+        <v>1.08440780639648</v>
       </c>
       <c r="U39">
-        <v>0.677026748657227</v>
+        <v>-1.30270195007324</v>
       </c>
       <c r="V39">
-        <v>0.364997863769531</v>
+        <v>3.44711112976074</v>
       </c>
     </row>
     <row r="40" ht="19.5" customHeight="1">
       <c r="A40" s="2">
-        <v>46195</v>
+        <v>46210</v>
       </c>
       <c r="B40">
-        <v>0.0426826477050781</v>
+        <v>-0.375518798828125</v>
       </c>
       <c r="C40">
-        <v>-1.65852737426758</v>
+        <v>-1.15375328063965</v>
       </c>
       <c r="D40">
-        <v>-1.5693187713623</v>
+        <v>-1.03360176086426</v>
       </c>
       <c r="E40">
-        <v>22.2600002288818</v>
+        <v>21.4899997711182</v>
       </c>
       <c r="F40">
-        <v>22.75</v>
+        <v>21.9549999237061</v>
       </c>
       <c r="G40">
-        <v>21.9200000762939</v>
+        <v>21.3250007629395</v>
       </c>
       <c r="H40">
-        <v>22.5200004577637</v>
+        <v>21.6900005340576</v>
       </c>
       <c r="I40">
-        <v>22.9673252105713</v>
+        <v>21.8200778961182</v>
       </c>
       <c r="J40">
-        <v>22.6023254394531</v>
+        <v>21.0972957611084</v>
       </c>
       <c r="K40">
-        <v>16162300</v>
+        <v>7265900</v>
       </c>
       <c r="L40">
-        <v>-0.0330952219665051</v>
+        <v>0.0607143566012383</v>
       </c>
       <c r="M40">
-        <v>28.1615428924561</v>
+        <v>31.316614151001</v>
       </c>
       <c r="N40">
-        <v>-8.91159534454346</v>
+        <v>-5.85662317276001</v>
       </c>
       <c r="O40" t="s">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="P40">
-        <v>-16.1065483093262</v>
+        <v>7.77024745941162</v>
       </c>
       <c r="Q40">
-        <v>22.9471015930176</v>
+        <v>21.6503143310547</v>
       </c>
       <c r="R40">
-        <v>22.89377784729</v>
+        <v>21.8759937286377</v>
       </c>
       <c r="S40">
-        <v>23.8384037017822</v>
+        <v>22.630199432373</v>
       </c>
       <c r="T40">
-        <v>0.217325210571289</v>
+        <v>-0.134922027587891</v>
       </c>
       <c r="U40">
-        <v>0.68232536315918</v>
+        <v>-0.227705001831055</v>
       </c>
       <c r="V40">
-        <v>0.364999771118164</v>
+        <v>0.722782135009766</v>
       </c>
     </row>
     <row r="41" ht="19.5" customHeight="1">
       <c r="A41" s="2">
-        <v>46191</v>
+        <v>46209</v>
       </c>
       <c r="B41">
-        <v>-0.0056915283203125</v>
+        <v>-0.518081665039063</v>
       </c>
       <c r="C41">
-        <v>-1.54353141784668</v>
+        <v>-1.2119312286377</v>
       </c>
       <c r="D41">
-        <v>-1.34329605102539</v>
+        <v>-1.10026741027832</v>
       </c>
       <c r="E41">
-        <v>22.7299995422363</v>
+        <v>21.7199993133545</v>
       </c>
       <c r="F41">
-        <v>23.1200008392334</v>
+        <v>21.7199993133545</v>
       </c>
       <c r="G41">
-        <v>22.6350002288818</v>
+        <v>21.4099998474121</v>
       </c>
       <c r="H41">
-        <v>22.7999992370605</v>
+        <v>21.4899997711182</v>
       </c>
       <c r="I41">
-        <v>23.367956161499</v>
+        <v>21.8874111175537</v>
       </c>
       <c r="J41">
-        <v>22.7519092559814</v>
+        <v>20.5938625335693</v>
       </c>
       <c r="K41">
-        <v>8352200</v>
+        <v>6209900</v>
       </c>
       <c r="L41">
-        <v>-0.0626190751791</v>
+        <v>0.00357146491296589</v>
       </c>
       <c r="M41">
-        <v>30.9167156219482</v>
+        <v>33.2648086547852</v>
       </c>
       <c r="N41">
-        <v>10.2793388366699</v>
+        <v>-9.78374195098877</v>
       </c>
       <c r="O41" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="P41">
-        <v>17.1931762695313</v>
+        <v>-13.5685234069824</v>
       </c>
       <c r="Q41">
-        <v>23.195686340332</v>
+        <v>21.7651062011719</v>
       </c>
       <c r="R41">
-        <v>23.2134113311768</v>
+        <v>21.9957885742188</v>
       </c>
       <c r="S41">
-        <v>24.0960483551025</v>
+        <v>22.7744026184082</v>
       </c>
       <c r="T41">
-        <v>0.247955322265625</v>
+        <v>0.167411804199219</v>
       </c>
       <c r="U41">
-        <v>0.116909027099609</v>
+        <v>-0.816137313842773</v>
       </c>
       <c r="V41">
-        <v>0.616046905517578</v>
+        <v>1.29354858398438</v>
       </c>
     </row>
     <row r="42" ht="19.5" customHeight="1">
       <c r="A42" s="2">
-        <v>46190</v>
+        <v>46205</v>
       </c>
       <c r="B42">
-        <v>-0.199920654296875</v>
+        <v>-0.419429779052734</v>
       </c>
       <c r="C42">
-        <v>-1.40483093261719</v>
+        <v>-0.915922164916992</v>
       </c>
       <c r="D42">
-        <v>-1.22029113769531</v>
+        <v>-1.01813888549805</v>
       </c>
       <c r="E42">
-        <v>22.3899993896484</v>
+        <v>22.0599994659424</v>
       </c>
       <c r="F42">
-        <v>23.8349990844727</v>
+        <v>22.5849990844727</v>
       </c>
       <c r="G42">
-        <v>22.3199996948242</v>
+        <v>21.7350006103516</v>
       </c>
       <c r="H42">
-        <v>23.5400009155273</v>
+        <v>22.0400009155273</v>
       </c>
       <c r="I42">
-        <v>24.3365993499756</v>
+        <v>22.1091861724854</v>
       </c>
       <c r="J42">
-        <v>23.4901847839355</v>
+        <v>21.7441864013672</v>
       </c>
       <c r="K42">
-        <v>13159400</v>
+        <v>9001800</v>
       </c>
       <c r="L42">
-        <v>-0.0621428713202477</v>
+        <v>0.00547617953270674</v>
       </c>
       <c r="M42">
-        <v>28.034912109375</v>
+        <v>36.8722991943359</v>
       </c>
       <c r="N42">
-        <v>-29.4497318267822</v>
+        <v>-19.0741996765137</v>
       </c>
       <c r="O42" t="s">
         <v>1</v>
       </c>
       <c r="P42">
-        <v>48.5132522583008</v>
+        <v>9.51707172393799</v>
       </c>
       <c r="Q42">
-        <v>23.419734954834</v>
+        <v>22.2072486877441</v>
       </c>
       <c r="R42">
-        <v>23.4456481933594</v>
+        <v>22.3150157928467</v>
       </c>
       <c r="S42">
-        <v>24.3058204650879</v>
+        <v>22.9963321685791</v>
       </c>
       <c r="T42">
-        <v>0.50160026550293</v>
+        <v>-0.475812911987305</v>
       </c>
       <c r="U42">
-        <v>1.17018508911133</v>
+        <v>0.009185791015625</v>
       </c>
       <c r="V42">
-        <v>0.846414566040039</v>
+        <v>0.364999771118164</v>
       </c>
     </row>
     <row r="43" ht="19.5" customHeight="1">
       <c r="A43" s="2">
-        <v>46189</v>
+        <v>46204</v>
       </c>
       <c r="B43">
-        <v>-1.51326751708984</v>
+        <v>-0.405847549438477</v>
       </c>
       <c r="C43">
-        <v>-1.97944068908691</v>
+        <v>-0.976701736450195</v>
       </c>
       <c r="D43">
-        <v>-1.50149154663086</v>
+        <v>-1.17591094970703</v>
       </c>
       <c r="E43">
-        <v>22.5300006866455</v>
+        <v>22.3500003814697</v>
       </c>
       <c r="F43">
-        <v>22.7199993133545</v>
+        <v>22.5499992370605</v>
       </c>
       <c r="G43">
-        <v>22.3549995422363</v>
+        <v>22.0102996826172</v>
       </c>
       <c r="H43">
-        <v>22.5699996948242</v>
+        <v>22.3199996948242</v>
       </c>
       <c r="I43">
-        <v>22.8074836730957</v>
+        <v>22.6419010162354</v>
       </c>
       <c r="J43">
-        <v>22.4424819946289</v>
+        <v>22.0874977111816</v>
       </c>
       <c r="K43">
-        <v>7550500</v>
+        <v>7270600</v>
       </c>
       <c r="L43">
-        <v>-0.129761919379234</v>
+        <v>0.00357137410901487</v>
       </c>
       <c r="M43">
-        <v>39.7374992370605</v>
+        <v>45.5630950927734</v>
       </c>
       <c r="N43">
-        <v>-12.3877696990967</v>
+        <v>-19.3071174621582</v>
       </c>
       <c r="O43" t="s">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="P43">
-        <v>-41.0672569274902</v>
+        <v>1.26358222961426</v>
       </c>
       <c r="Q43">
-        <v>23.05029296875</v>
+        <v>22.4488906860352</v>
       </c>
       <c r="R43">
-        <v>23.3773975372314</v>
+        <v>22.4495525360107</v>
       </c>
       <c r="S43">
-        <v>24.384105682373</v>
+        <v>23.1492938995361</v>
       </c>
       <c r="T43">
-        <v>0.0874843597412109</v>
+        <v>0.0919017791748047</v>
       </c>
       <c r="U43">
-        <v>0.0874824523925781</v>
+        <v>0.0771980285644531</v>
       </c>
       <c r="V43">
-        <v>0.365001678466797</v>
+        <v>0.554403305053711</v>
       </c>
     </row>
     <row r="44" ht="19.5" customHeight="1">
       <c r="A44" s="2">
-        <v>46188</v>
+        <v>46203</v>
       </c>
       <c r="B44">
-        <v>-1.77403259277344</v>
+        <v>-0.683012008666992</v>
       </c>
       <c r="C44">
-        <v>-1.58996772766113</v>
+        <v>-0.766977310180664</v>
       </c>
       <c r="D44">
-        <v>-1.15474510192871</v>
+        <v>-1.12672424316406</v>
       </c>
       <c r="E44">
-        <v>23.0599994659424</v>
+        <v>22.6000003814697</v>
       </c>
       <c r="F44">
-        <v>23.1299991607666</v>
+        <v>22.7000007629395</v>
       </c>
       <c r="G44">
-        <v>22.4850006103516</v>
+        <v>21.9599990844727</v>
       </c>
       <c r="H44">
-        <v>22.5599994659424</v>
+        <v>22.0900001525879</v>
       </c>
       <c r="I44">
-        <v>22.7412891387939</v>
+        <v>23.2584552764893</v>
       </c>
       <c r="J44">
-        <v>21.392599105835</v>
+        <v>20.9772338867188</v>
       </c>
       <c r="K44">
-        <v>12916000</v>
+        <v>4630600</v>
       </c>
       <c r="L44">
-        <v>-0.165476113557816</v>
+        <v>0.0226190648972988</v>
       </c>
       <c r="M44">
-        <v>45.3561096191406</v>
+        <v>56.4648246765137</v>
       </c>
       <c r="N44">
-        <v>1.39943420886993</v>
+        <v>35.7507209777832</v>
       </c>
       <c r="O44" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="P44">
-        <v>-100.000007629395</v>
+        <v>-35.5566825866699</v>
       </c>
       <c r="Q44">
-        <v>23.4940910339355</v>
+        <v>22.5476150512695</v>
       </c>
       <c r="R44">
-        <v>23.88987159729</v>
+        <v>22.6672439575195</v>
       </c>
       <c r="S44">
-        <v>24.7133960723877</v>
+        <v>23.3205070495605</v>
       </c>
       <c r="T44">
-        <v>-0.388710021972656</v>
+        <v>0.558454513549805</v>
       </c>
       <c r="U44">
-        <v>-1.0924015045166</v>
+        <v>-0.982765197753906</v>
       </c>
       <c r="V44">
-        <v>1.34869003295898</v>
+        <v>2.28122138977051</v>
+      </c>
+    </row>
+    <row r="45" ht="19.5" customHeight="1">
+      <c r="A45" s="2">
+        <v>46202</v>
+      </c>
+      <c r="B45">
+        <v>-0.565788269042969</v>
+      </c>
+      <c r="C45">
+        <v>-0.206932067871094</v>
+      </c>
+      <c r="D45">
+        <v>-0.893896102905273</v>
+      </c>
+      <c r="E45">
+        <v>22.8600006103516</v>
+      </c>
+      <c r="F45">
+        <v>23.4799995422363</v>
+      </c>
+      <c r="G45">
+        <v>22.5149993896484</v>
+      </c>
+      <c r="H45">
+        <v>22.5499992370605</v>
+      </c>
+      <c r="I45">
+        <v>22.7034931182861</v>
+      </c>
+      <c r="J45">
+        <v>21.9739532470703</v>
+      </c>
+      <c r="K45">
+        <v>16043900</v>
+      </c>
+      <c r="L45">
+        <v>0.0426190681755543</v>
+      </c>
+      <c r="M45">
+        <v>41.5944938659668</v>
+      </c>
+      <c r="N45">
+        <v>28.7921371459961</v>
+      </c>
+      <c r="O45" t="s">
+        <v>21</v>
+      </c>
+      <c r="P45">
+        <v>-20.1520481109619</v>
+      </c>
+      <c r="Q45">
+        <v>22.988452911377</v>
+      </c>
+      <c r="R45">
+        <v>23.0405597686768</v>
+      </c>
+      <c r="S45">
+        <v>23.5438270568848</v>
+      </c>
+      <c r="T45">
+        <v>-0.776506423950195</v>
+      </c>
+      <c r="U45">
+        <v>-0.541046142578125</v>
+      </c>
+      <c r="V45">
+        <v>0.72953987121582</v>
       </c>
     </row>
   </sheetData>

</xml_diff>